<commit_message>
Adding Finance with Excel Test
</commit_message>
<xml_diff>
--- a/Excel-Finance/JLoka-Finance-01.xlsx
+++ b/Excel-Finance/JLoka-Finance-01.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\books-and-tutorials\Finance-Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12BE2EAF-E0BF-4D0D-8916-8CB057BD4984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4068D8DE-841B-42E7-867C-CD60AC7B5A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="74">
   <si>
     <t>Sunday</t>
   </si>
@@ -127,6 +130,138 @@
   </si>
   <si>
     <t>CountIf</t>
+  </si>
+  <si>
+    <t>ITEM</t>
+  </si>
+  <si>
+    <t>PRICE</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Week 2</t>
+  </si>
+  <si>
+    <t>REVENUE</t>
+  </si>
+  <si>
+    <t>% of Revenue</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>REGION</t>
+  </si>
+  <si>
+    <t>PRODUCT</t>
+  </si>
+  <si>
+    <t>SALES</t>
+  </si>
+  <si>
+    <t>NORTH</t>
+  </si>
+  <si>
+    <t>SOUTH</t>
+  </si>
+  <si>
+    <t>EAST</t>
+  </si>
+  <si>
+    <t>WEST</t>
+  </si>
+  <si>
+    <t>PRODUCT A</t>
+  </si>
+  <si>
+    <t>PRODUCT B</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>INVESTOR_ID</t>
+  </si>
+  <si>
+    <t>INVESTOR_NAME</t>
+  </si>
+  <si>
+    <t>COMPANY_NAME</t>
+  </si>
+  <si>
+    <t>INVESTMENT AMOUNT (USD)</t>
+  </si>
+  <si>
+    <t>INVESTMENT_DATE</t>
+  </si>
+  <si>
+    <t>INV-001</t>
+  </si>
+  <si>
+    <t>INV-002</t>
+  </si>
+  <si>
+    <t>INV-003</t>
+  </si>
+  <si>
+    <t>INV-004</t>
+  </si>
+  <si>
+    <t>INV-005</t>
+  </si>
+  <si>
+    <t>INV-006</t>
+  </si>
+  <si>
+    <t>INV-007</t>
+  </si>
+  <si>
+    <t>INV-008</t>
+  </si>
+  <si>
+    <t>Jafar Loka-01</t>
+  </si>
+  <si>
+    <t>Jafar Loka-02</t>
+  </si>
+  <si>
+    <t>Jafar Loka-03</t>
+  </si>
+  <si>
+    <t>Jafar Loka-04</t>
+  </si>
+  <si>
+    <t>Jafar Loka-05</t>
+  </si>
+  <si>
+    <t>Jafar Loka-06</t>
+  </si>
+  <si>
+    <t>Jafar Loka-07</t>
+  </si>
+  <si>
+    <t>Jafar Loka-08</t>
   </si>
 </sst>
 </file>
@@ -135,7 +270,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -175,7 +310,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -224,8 +359,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -258,6 +417,303 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color theme="2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color theme="2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -267,7 +723,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -278,10 +734,25 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="2" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -293,24 +764,80 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="9"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="9" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -319,6 +846,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF0000"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -780,243 +1312,258 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11" t="s">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11" t="s">
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="12">
+      <c r="A3" s="23">
         <v>46144</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="14">
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="25">
         <v>250.25</v>
       </c>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="N3" s="17" t="s">
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="N3" s="11" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="12">
+      <c r="A4" s="23">
         <v>46145</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="14">
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="25">
         <v>300</v>
       </c>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="15">
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="21">
         <f>(E4-E3)/E3</f>
         <v>0.19880119880119881</v>
       </c>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="N4" s="16">
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="N4" s="10">
         <f>AVERAGE(I4:L11)</f>
         <v>-8.1596436336491718E-2</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="12">
+      <c r="A5" s="23">
         <v>46146</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="14">
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="25">
         <v>350.15</v>
       </c>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="15">
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="21">
         <f>(E5-E4)/E4</f>
         <v>0.1671666666666666</v>
       </c>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
+      <c r="A6" s="23">
         <v>46147</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="14">
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="25">
         <v>650.5</v>
       </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="15">
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="21">
         <f>(E6-E5)/E5</f>
         <v>0.85777523918320731</v>
       </c>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="N6" s="17" t="s">
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="N6" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
+      <c r="A7" s="23">
         <v>46148</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="14">
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="25">
         <v>600.35</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="15">
-        <f t="shared" ref="I5:I10" si="0">(E7-E6)/E6</f>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="21">
+        <f t="shared" ref="I7:I10" si="0">(E7-E6)/E6</f>
         <v>-7.7094542659492657E-2</v>
       </c>
-      <c r="J7" s="15"/>
-      <c r="K7" s="15"/>
-      <c r="L7" s="15"/>
-      <c r="N7" s="18" t="str">
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
+      <c r="L7" s="21"/>
+      <c r="N7" s="12" t="str">
         <f>IF(N4&gt;0,"Positive","Negative")</f>
         <v>Negative</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
+      <c r="A8" s="23">
         <v>46149</v>
       </c>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="14">
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="25">
         <v>150.19999999999999</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="15">
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="25"/>
+      <c r="I8" s="21">
         <f t="shared" si="0"/>
         <v>-0.74981260931123517</v>
       </c>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
+      <c r="J8" s="21"/>
+      <c r="K8" s="21"/>
+      <c r="L8" s="21"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="12">
+      <c r="A9" s="23">
         <v>46150</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="14">
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="25">
         <v>55.5</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15">
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="21">
         <f t="shared" si="0"/>
         <v>-0.6304926764314247</v>
       </c>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="21"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
+      <c r="A10" s="23">
         <v>46151</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="14">
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="25">
         <v>80.5</v>
       </c>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15">
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="21">
         <f t="shared" si="0"/>
         <v>0.45045045045045046</v>
       </c>
-      <c r="J10" s="15"/>
-      <c r="K10" s="15"/>
-      <c r="L10" s="15"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="12">
+      <c r="A11" s="23">
         <v>46152</v>
       </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="14">
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="25">
         <v>10.5</v>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15">
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="21">
         <f t="shared" ref="I11" si="1">(E11-E10)/E10</f>
         <v>-0.86956521739130432</v>
       </c>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15"/>
+      <c r="J11" s="21"/>
+      <c r="K11" s="21"/>
+      <c r="L11" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A7:D7"/>
     <mergeCell ref="I10:L10"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A11:D11"/>
@@ -1033,21 +1580,6 @@
     <mergeCell ref="I9:L9"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="E6:H6"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A7:D7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1061,245 +1593,900 @@
     <col min="2" max="2" width="13.42578125" customWidth="1"/>
     <col min="3" max="3" width="30.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="24"/>
-      <c r="E2" s="19" t="s">
+      <c r="D2" s="18"/>
+      <c r="E2" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="16" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="20">
+      <c r="B3" s="14">
         <v>46144</v>
       </c>
-      <c r="C3" s="21">
+      <c r="C3" s="15">
         <v>1000000</v>
       </c>
-      <c r="D3" s="23"/>
-      <c r="E3" s="26">
+      <c r="D3" s="17"/>
+      <c r="E3" s="20">
         <f>SUM(C3:C17)</f>
         <v>1653820000</v>
       </c>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
+      <c r="F3" s="20">
+        <f>MAX(C3:C17)</f>
+        <v>800000000</v>
+      </c>
+      <c r="G3" s="20">
+        <f>MIN(C3:C17)</f>
+        <v>10000</v>
+      </c>
+      <c r="H3" s="19">
+        <f>COUNT(C3:C17)</f>
+        <v>15</v>
+      </c>
+      <c r="I3" s="19">
+        <f>COUNTIF(C3:C17,"&gt;1000000")</f>
+        <v>8</v>
+      </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="20">
+      <c r="B4" s="14">
         <v>46145</v>
       </c>
-      <c r="C4" s="21">
+      <c r="C4" s="15">
         <v>2000000</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
+      <c r="D4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="20">
+      <c r="B5" s="14">
         <v>46146</v>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="15">
         <v>3000000</v>
       </c>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="20">
+      <c r="B6" s="14">
         <v>46147</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="15">
         <v>10000</v>
       </c>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="20">
+      <c r="B7" s="14">
         <v>46148</v>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="15">
         <v>100000</v>
       </c>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="20">
+      <c r="B8" s="14">
         <v>46149</v>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="15">
         <v>500000</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="20">
+      <c r="B9" s="14">
         <v>46150</v>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="15">
         <v>6000000</v>
       </c>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="20">
+      <c r="B10" s="14">
         <v>46151</v>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="15">
         <v>100000000</v>
       </c>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="20">
+      <c r="B11" s="14">
         <v>46152</v>
       </c>
-      <c r="C11" s="21">
+      <c r="C11" s="15">
         <v>700000000</v>
       </c>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="20">
+      <c r="B12" s="14">
         <v>46153</v>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="15">
         <v>800000000</v>
       </c>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="20">
+      <c r="B13" s="14">
         <v>46154</v>
       </c>
-      <c r="C13" s="21">
+      <c r="C13" s="15">
         <v>10000</v>
       </c>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="20">
+      <c r="B14" s="14">
         <v>46155</v>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="15">
         <v>300000</v>
       </c>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="20">
+      <c r="B15" s="14">
         <v>46156</v>
       </c>
-      <c r="C15" s="21">
+      <c r="C15" s="15">
         <v>15000000</v>
       </c>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="20">
+      <c r="B16" s="14">
         <v>46157</v>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="15">
         <v>25000000</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="20">
+      <c r="B17" s="14">
         <v>46158</v>
       </c>
-      <c r="C17" s="21">
+      <c r="C17" s="15">
         <v>900000</v>
       </c>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D44A967B-77A0-46E6-9D75-84A934B0FAA8}">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="28" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="F1" s="28"/>
+      <c r="G1" s="27" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="27"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="32">
+        <f ca="1">RANDBETWEEN(10, 50)</f>
+        <v>41</v>
+      </c>
+      <c r="C3" s="38">
+        <f ca="1">RANDBETWEEN(2, 10)</f>
+        <v>6</v>
+      </c>
+      <c r="D3" s="30">
+        <f ca="1">RANDBETWEEN(2, 10)</f>
+        <v>8</v>
+      </c>
+      <c r="E3" s="37">
+        <f ca="1">$B3*C3</f>
+        <v>246</v>
+      </c>
+      <c r="F3" s="44">
+        <f ca="1">$B3*D3</f>
+        <v>328</v>
+      </c>
+      <c r="G3" s="47">
+        <f ca="1">(E3+F3)/(E$8+F$8)</f>
+        <v>0.25879170423805231</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="32">
+        <f t="shared" ref="B4:B7" ca="1" si="0">RANDBETWEEN(10, 50)</f>
+        <v>40</v>
+      </c>
+      <c r="C4" s="39">
+        <f t="shared" ref="C4:D7" ca="1" si="1">RANDBETWEEN(2, 10)</f>
+        <v>10</v>
+      </c>
+      <c r="D4" s="33">
+        <f t="shared" ca="1" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="E4" s="37">
+        <f t="shared" ref="E4:F7" ca="1" si="2">$B4*C4</f>
+        <v>400</v>
+      </c>
+      <c r="F4" s="45">
+        <f t="shared" ca="1" si="2"/>
+        <v>200</v>
+      </c>
+      <c r="G4" s="47">
+        <f ca="1">(E4+F4)/(E$8+F$8)</f>
+        <v>0.27051397655545534</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="32">
+        <f t="shared" ca="1" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="C5" s="39">
+        <f t="shared" ca="1" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="D5" s="36">
+        <f t="shared" ca="1" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="E5" s="37">
+        <f t="shared" ca="1" si="2"/>
+        <v>192</v>
+      </c>
+      <c r="F5" s="44">
+        <f t="shared" ca="1" si="2"/>
+        <v>72</v>
+      </c>
+      <c r="G5" s="47">
+        <f t="shared" ref="G5:G7" ca="1" si="3">(E5+F5)/(E$8+F$8)</f>
+        <v>0.11902614968440037</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="32">
+        <f t="shared" ca="1" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C6" s="34">
+        <f t="shared" ca="1" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="D6" s="33">
+        <f t="shared" ca="1" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="E6" s="37">
+        <f t="shared" ca="1" si="2"/>
+        <v>60</v>
+      </c>
+      <c r="F6" s="44">
+        <f t="shared" ca="1" si="2"/>
+        <v>60</v>
+      </c>
+      <c r="G6" s="47">
+        <f t="shared" ca="1" si="3"/>
+        <v>5.4102795311091072E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="C7" s="40">
+        <f t="shared" ca="1" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="D7" s="35">
+        <f t="shared" ca="1" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="E7" s="37">
+        <f t="shared" ca="1" si="2"/>
+        <v>220</v>
+      </c>
+      <c r="F7" s="44">
+        <f t="shared" ca="1" si="2"/>
+        <v>440</v>
+      </c>
+      <c r="G7" s="47">
+        <f t="shared" ca="1" si="3"/>
+        <v>0.29756537421100088</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="43"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="46">
+        <f ca="1">SUM(E3:E7)</f>
+        <v>1118</v>
+      </c>
+      <c r="F8" s="46">
+        <f ca="1">SUM(F3:F7)</f>
+        <v>1100</v>
+      </c>
+      <c r="G8" s="43"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C9" s="42"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="G1:G2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A353DF0-38D4-4363-880C-1DE1AFCD6401}">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="49" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="49"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="61" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="57" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="51">
+        <f ca="1">RANDBETWEEN(500, 1000)</f>
+        <v>811</v>
+      </c>
+      <c r="F2" s="55" t="s">
+        <v>48</v>
+      </c>
+      <c r="G2" s="56">
+        <f ca="1">SUMIF($A$2:$A$9, F2, $C$2:$C$9)</f>
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="63" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="59" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" s="54">
+        <f t="shared" ref="C3:C9" ca="1" si="0">RANDBETWEEN(500, 1000)</f>
+        <v>688</v>
+      </c>
+      <c r="F3" s="43" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" s="43">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F3)</f>
+        <v>721</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="62" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="58" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="54">
+        <f t="shared" ca="1" si="0"/>
+        <v>706</v>
+      </c>
+      <c r="F4" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" s="43">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F4)</f>
+        <v>952</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="63" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="59" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="54">
+        <f t="shared" ca="1" si="0"/>
+        <v>680</v>
+      </c>
+      <c r="F5" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="56">
+        <f ca="1">SUMIF($A$2:$A$9, F5, $C$2:$C$9)</f>
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="58" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="54">
+        <f t="shared" ca="1" si="0"/>
+        <v>721</v>
+      </c>
+      <c r="F6" s="43" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="43">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F6)</f>
+        <v>811</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="63" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="59" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="54">
+        <f t="shared" ca="1" si="0"/>
+        <v>952</v>
+      </c>
+      <c r="F7" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" s="43">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F7)</f>
+        <v>688</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="62" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="58" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="54">
+        <f t="shared" ca="1" si="0"/>
+        <v>646</v>
+      </c>
+      <c r="F8" s="55" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="56">
+        <f ca="1">SUMIF($A$2:$A$9, F8, $C$2:$C$9)</f>
+        <v>1386</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="64" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="60" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="52">
+        <f t="shared" ca="1" si="0"/>
+        <v>968</v>
+      </c>
+      <c r="F9" s="43" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="43">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F9)</f>
+        <v>706</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F10" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="43">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F10)</f>
+        <v>680</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F11" s="55" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="56">
+        <f ca="1">SUMIF($A$2:$A$9, F11, $C$2:$C$9)</f>
+        <v>1614</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F12" s="43" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" s="43">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F12)</f>
+        <v>646</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F13" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="G13" s="43">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F13)</f>
+        <v>968</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F14" s="50" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" s="53">
+        <f ca="1">SUM(G2,G5,G8,G11)</f>
+        <v>6172</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22AB70FF-96FA-4025-A517-8BDE3ECE5EBF}">
+  <dimension ref="B1:F9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12.7109375" style="65" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" style="65" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" style="65" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.28515625" style="65" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" style="65" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="B1" s="71" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="69" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="69" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="70" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="68" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="65" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="65" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="65" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" s="66">
+        <f ca="1">RANDBETWEEN(5000, 80000)</f>
+        <v>21206</v>
+      </c>
+      <c r="F2" s="67">
+        <f>DATE(2026, 5, 7)</f>
+        <v>46149</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="65" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="65" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="65" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="66">
+        <f t="shared" ref="E3:E9" ca="1" si="0">RANDBETWEEN(5000, 80000)</f>
+        <v>14031</v>
+      </c>
+      <c r="F3" s="67">
+        <f>DATE(2026, 6, 7)</f>
+        <v>46180</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="65" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="65" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="65" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="66">
+        <f t="shared" ca="1" si="0"/>
+        <v>14215</v>
+      </c>
+      <c r="F4" s="67">
+        <f>DATE(2026, 7, 7)</f>
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="65" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="65" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="65" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="66">
+        <f t="shared" ca="1" si="0"/>
+        <v>44607</v>
+      </c>
+      <c r="F5" s="67">
+        <f>DATE(2026, 8, 7)</f>
+        <v>46241</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="65" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="65" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="65" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" s="66">
+        <f t="shared" ca="1" si="0"/>
+        <v>64020</v>
+      </c>
+      <c r="F6" s="67">
+        <f>DATE(2026, 9, 7)</f>
+        <v>46272</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="65" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="66">
+        <f t="shared" ca="1" si="0"/>
+        <v>8305</v>
+      </c>
+      <c r="F7" s="67">
+        <f>DATE(2026, 10, 7)</f>
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="65" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="65" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="65" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="66">
+        <f t="shared" ca="1" si="0"/>
+        <v>8319</v>
+      </c>
+      <c r="F8" s="67">
+        <f>DATE(2026, 11, 7)</f>
+        <v>46333</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="65" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="65" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="65" t="s">
+        <v>73</v>
+      </c>
+      <c r="E9" s="66">
+        <f t="shared" ca="1" si="0"/>
+        <v>70353</v>
+      </c>
+      <c r="F9" s="67">
+        <f>DATE(2026, 12, 7)</f>
+        <v>46363</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adding Finance & Excel file
</commit_message>
<xml_diff>
--- a/Excel-Finance/JLoka-Finance-01.xlsx
+++ b/Excel-Finance/JLoka-Finance-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\books-and-tutorials\Finance-Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4068D8DE-841B-42E7-867C-CD60AC7B5A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F41F8F-04F6-40F5-BA6F-2BFC3A455D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,24 @@
     <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
     <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
     <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet8" sheetId="8" r:id="rId8"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet7!$B$1:$F$9</definedName>
+    <definedName name="Slicer_COMPANY_NAME">#N/A</definedName>
+    <definedName name="Slicer_INVESTMENT_AMOUNT__USD">#N/A</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
+      <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
+        <x14:slicerCache r:id="rId9"/>
+        <x14:slicerCache r:id="rId10"/>
+      </x15:slicerCaches>
+    </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
@@ -40,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="80">
   <si>
     <t>Sunday</t>
   </si>
@@ -262,17 +277,36 @@
   </si>
   <si>
     <t>Jafar Loka-08</t>
+  </si>
+  <si>
+    <t>SUM Of Investment Amount</t>
+  </si>
+  <si>
+    <t>JLoka Stock Returns</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Jloka-01</t>
+  </si>
+  <si>
+    <t>Jloka-02</t>
+  </si>
+  <si>
+    <t>Jloka-03</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -305,6 +339,14 @@
       <b/>
       <sz val="11"/>
       <color theme="5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -723,7 +765,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -749,30 +791,6 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -788,7 +806,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -799,13 +816,10 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="9" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="44" fontId="0" fillId="9" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -820,23 +834,74 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -844,7 +909,208 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -860,6 +1126,1436 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1320" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="95000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:effectLst>
+                  <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                    <a:prstClr val="black">
+                      <a:alpha val="40000"/>
+                    </a:prstClr>
+                  </a:outerShdw>
+                </a:effectLst>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Stock Returns</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1320" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="34925" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet8!$B$4:$B$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>2011</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2012</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2013</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2014</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2015</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2016</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2017</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2018</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2021</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet8!$C$4:$C$14</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>0.74632334827253011</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.96726538064451084</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.34234357821502415</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.6802225754616299</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.41154429073134569</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.8166285419759518E-3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.55602648328598325</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.72204098578482745</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.75989775807371251</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36214243666635559</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8.0557715692428644E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9F87-4B16-9178-53052F6E00C5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln w="34925" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet8!$B$4:$B$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>2011</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2012</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2013</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2014</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2015</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2016</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2017</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2018</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2021</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet8!$D$4:$D$14</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>7.6764236190715374E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5.4354528886120357E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.28344606593773036</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.71322647348581636</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.24424704666357588</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9.6777844968651827E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.52020423431596585</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.32085133206821126</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.47604524511131241</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.96824967018629216</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.99040654877882894</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-9F87-4B16-9178-53052F6E00C5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:spPr>
+            <a:ln w="34925" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet8!$B$4:$B$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>2011</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2012</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2013</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2014</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2015</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2016</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2017</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2018</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2021</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet8!$E$4:$E$14</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>0.59766622878496245</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.35034220588725351</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.69553741865844598</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.58331324969536502</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.5648847882053256E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.70430520884159553</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.34173611134409643</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.38026533146699537</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.61216195487650615</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.94629380652869344</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.8497834350972423</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-9F87-4B16-9178-53052F6E00C5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1734618992"/>
+        <c:axId val="1734630512"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1734618992"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+                <a:alpha val="10000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1734630512"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1734630512"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                  <a:alpha val="10000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1734618992"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="85000"/>
+            <a:lumOff val="15000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="1100" b="1"/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="233">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="85000"/>
+              <a:lumOff val="15000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="34925" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="5000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="95000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:defRPr>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer" Requires="sle15">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="COMPANY_NAME">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{667605D0-8334-FF95-FC58-ECB955FC2ED6}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="COMPANY_NAME"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="10277475" y="66675"/>
+              <a:ext cx="1828800" cy="2524125"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This shape represents a table slicer. Table slicers are not supported in this version of Excel.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2007 or earlier, the slicer can't be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer" Requires="sle15">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="3" name="INVESTMENT AMOUNT (USD)">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34C2D707-DCB3-41FC-EB4C-25614133E04E}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="INVESTMENT AMOUNT (USD)"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="8286750" y="76200"/>
+              <a:ext cx="1828800" cy="2524125"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This shape represents a table slicer. Table slicers are not supported in this version of Excel.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2007 or earlier, the slicer can't be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>85725</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D179C9A-3D96-A297-DF2A-3741166D9F0E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_COMPANY_NAME" xr10:uid="{01C3EAA2-3CA2-48B6-8C0C-A74C74C9E24D}" sourceName="COMPANY_NAME">
+  <extLst>
+    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{2F2917AC-EB37-4324-AD4E-5DD8C200BD13}">
+      <x15:tableSlicerCache tableId="2" column="3"/>
+    </x:ext>
+  </extLst>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache2.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_INVESTMENT_AMOUNT__USD" xr10:uid="{6D3F0E70-2139-4563-812F-FA2D0194416E}" sourceName="INVESTMENT AMOUNT (USD)">
+  <extLst>
+    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{2F2917AC-EB37-4324-AD4E-5DD8C200BD13}">
+      <x15:tableSlicerCache tableId="2" column="4"/>
+    </x:ext>
+  </extLst>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
+  <slicer name="COMPANY_NAME" xr10:uid="{D2D1BF6C-F74D-49B7-A9DD-B6FC782BA13F}" cache="Slicer_COMPANY_NAME" caption="COMPANY_NAME" rowHeight="241300"/>
+  <slicer name="INVESTMENT AMOUNT (USD)" xr10:uid="{3A768713-1BDF-4D4C-9D8A-AFB79056E964}" cache="Slicer_INVESTMENT_AMOUNT__USD" caption="INVESTMENT AMOUNT (USD)" rowHeight="241300"/>
+</slicers>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{385DC015-9960-47FA-A637-6B66C3CB4FFA}" name="JLoka_Investors" displayName="JLoka_Investors" ref="B1:F9" totalsRowShown="0" dataDxfId="5" tableBorderDxfId="11">
+  <autoFilter ref="B1:F9" xr:uid="{22AB70FF-96FA-4025-A517-8BDE3ECE5EBF}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Jafar Loka-01"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{0BE1A407-37E2-45E1-A4B9-6EE27C852CA8}" name="INVESTOR_ID" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{F40E02B0-B4B8-4130-A683-00045FEF2BC6}" name="INVESTOR_NAME" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{EB541472-54EA-4246-959A-8F16F8FDA58F}" name="COMPANY_NAME" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{B149ED9E-81EF-4313-90DA-EDCF3ACBE03C}" name="INVESTMENT AMOUNT (USD)" dataDxfId="7" dataCellStyle="Currency"/>
+    <tableColumn id="5" xr3:uid="{5C700949-A13F-423E-81D1-C89753142DF7}" name="INVESTMENT_DATE" dataDxfId="6"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E0111534-CC78-4AAC-9FB0-08AB9DCECE24}" name="Table4" displayName="Table4" ref="B3:E14" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" dataCellStyle="Percent">
+  <autoFilter ref="B3:E14" xr:uid="{E0111534-CC78-4AAC-9FB0-08AB9DCECE24}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{B5AEA49B-906B-4BA3-9E02-DF265E516312}" name="Year"/>
+    <tableColumn id="2" xr3:uid="{8C94788E-9FB3-46B0-A805-B97EFDDC36C5}" name="Jloka-01" dataDxfId="4" dataCellStyle="Percent">
+      <calculatedColumnFormula>RAND()</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{A2693482-C7C8-4B05-9865-B12ABE5CC110}" name="Jloka-02" dataDxfId="3" dataCellStyle="Percent">
+      <calculatedColumnFormula>RAND()</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{8F26A52C-2531-497C-A839-2A770D581E4E}" name="Jloka-03" dataDxfId="2" dataCellStyle="Percent">
+      <calculatedColumnFormula>RAND()</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1312,258 +3008,243 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26" t="s">
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26" t="s">
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="23">
+      <c r="A3" s="57">
         <v>46144</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25">
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="59">
         <v>250.25</v>
       </c>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="58"/>
+      <c r="L3" s="58"/>
       <c r="N3" s="11" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="23">
+      <c r="A4" s="57">
         <v>46145</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="25">
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="59">
         <v>300</v>
       </c>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="21">
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="60">
         <f>(E4-E3)/E3</f>
         <v>0.19880119880119881</v>
       </c>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
+      <c r="J4" s="60"/>
+      <c r="K4" s="60"/>
+      <c r="L4" s="60"/>
       <c r="N4" s="10">
         <f>AVERAGE(I4:L11)</f>
         <v>-8.1596436336491718E-2</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="23">
+      <c r="A5" s="57">
         <v>46146</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="25">
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="59">
         <v>350.15</v>
       </c>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="21">
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="60">
         <f>(E5-E4)/E4</f>
         <v>0.1671666666666666</v>
       </c>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="21"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="60"/>
+      <c r="L5" s="60"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="23">
+      <c r="A6" s="57">
         <v>46147</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="25">
+      <c r="B6" s="58"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="59">
         <v>650.5</v>
       </c>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="21">
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
+      <c r="H6" s="59"/>
+      <c r="I6" s="60">
         <f>(E6-E5)/E5</f>
         <v>0.85777523918320731</v>
       </c>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
+      <c r="J6" s="60"/>
+      <c r="K6" s="60"/>
+      <c r="L6" s="60"/>
       <c r="N6" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="23">
+      <c r="A7" s="57">
         <v>46148</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="25">
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="59">
         <v>600.35</v>
       </c>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="21">
+      <c r="F7" s="59"/>
+      <c r="G7" s="59"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="60">
         <f t="shared" ref="I7:I10" si="0">(E7-E6)/E6</f>
         <v>-7.7094542659492657E-2</v>
       </c>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
+      <c r="J7" s="60"/>
+      <c r="K7" s="60"/>
+      <c r="L7" s="60"/>
       <c r="N7" s="12" t="str">
         <f>IF(N4&gt;0,"Positive","Negative")</f>
         <v>Negative</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="23">
+      <c r="A8" s="57">
         <v>46149</v>
       </c>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="25">
+      <c r="B8" s="58"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="59">
         <v>150.19999999999999</v>
       </c>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="21">
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60">
         <f t="shared" si="0"/>
         <v>-0.74981260931123517</v>
       </c>
-      <c r="J8" s="21"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
+      <c r="J8" s="60"/>
+      <c r="K8" s="60"/>
+      <c r="L8" s="60"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="23">
+      <c r="A9" s="57">
         <v>46150</v>
       </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="25">
+      <c r="B9" s="58"/>
+      <c r="C9" s="58"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="59">
         <v>55.5</v>
       </c>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="21">
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="60">
         <f t="shared" si="0"/>
         <v>-0.6304926764314247</v>
       </c>
-      <c r="J9" s="21"/>
-      <c r="K9" s="21"/>
-      <c r="L9" s="21"/>
+      <c r="J9" s="60"/>
+      <c r="K9" s="60"/>
+      <c r="L9" s="60"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="23">
+      <c r="A10" s="57">
         <v>46151</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="25">
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="58"/>
+      <c r="E10" s="59">
         <v>80.5</v>
       </c>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="21">
+      <c r="F10" s="59"/>
+      <c r="G10" s="59"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="60">
         <f t="shared" si="0"/>
         <v>0.45045045045045046</v>
       </c>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
+      <c r="J10" s="60"/>
+      <c r="K10" s="60"/>
+      <c r="L10" s="60"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="23">
+      <c r="A11" s="57">
         <v>46152</v>
       </c>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="25">
+      <c r="B11" s="58"/>
+      <c r="C11" s="58"/>
+      <c r="D11" s="58"/>
+      <c r="E11" s="59">
         <v>10.5</v>
       </c>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="21">
+      <c r="F11" s="59"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="59"/>
+      <c r="I11" s="60">
         <f t="shared" ref="I11" si="1">(E11-E10)/E10</f>
         <v>-0.86956521739130432</v>
       </c>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21"/>
-      <c r="L11" s="21"/>
+      <c r="J11" s="60"/>
+      <c r="K11" s="60"/>
+      <c r="L11" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="E6:H6"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A7:D7"/>
     <mergeCell ref="I10:L10"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A11:D11"/>
@@ -1580,6 +3261,21 @@
     <mergeCell ref="I9:L9"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1851,7 +3547,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D44A967B-77A0-46E6-9D75-84A934B0FAA8}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="11" customWidth="1"/>
@@ -1860,205 +3556,202 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="62" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="63" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28" t="s">
+      <c r="D1" s="63"/>
+      <c r="E1" s="63" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="28"/>
-      <c r="G1" s="27" t="s">
+      <c r="F1" s="63"/>
+      <c r="G1" s="62" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="27"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="29" t="s">
+      <c r="A2" s="62"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E2" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="F2" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="27"/>
+      <c r="G2" s="62"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="32">
+      <c r="B3" s="24">
         <f ca="1">RANDBETWEEN(10, 50)</f>
-        <v>41</v>
-      </c>
-      <c r="C3" s="38">
+        <v>20</v>
+      </c>
+      <c r="C3" s="30">
         <f ca="1">RANDBETWEEN(2, 10)</f>
-        <v>6</v>
-      </c>
-      <c r="D3" s="30">
+        <v>3</v>
+      </c>
+      <c r="D3" s="22">
         <f ca="1">RANDBETWEEN(2, 10)</f>
         <v>8</v>
       </c>
-      <c r="E3" s="37">
+      <c r="E3" s="29">
         <f ca="1">$B3*C3</f>
-        <v>246</v>
-      </c>
-      <c r="F3" s="44">
+        <v>60</v>
+      </c>
+      <c r="F3" s="35">
         <f ca="1">$B3*D3</f>
-        <v>328</v>
-      </c>
-      <c r="G3" s="47">
+        <v>160</v>
+      </c>
+      <c r="G3" s="38">
         <f ca="1">(E3+F3)/(E$8+F$8)</f>
-        <v>0.25879170423805231</v>
+        <v>0.14996591683708249</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="32">
+      <c r="B4" s="24">
         <f t="shared" ref="B4:B7" ca="1" si="0">RANDBETWEEN(10, 50)</f>
+        <v>48</v>
+      </c>
+      <c r="C4" s="31">
+        <f t="shared" ref="C4:D7" ca="1" si="1">RANDBETWEEN(2, 10)</f>
+        <v>2</v>
+      </c>
+      <c r="D4" s="25">
+        <f t="shared" ca="1" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="E4" s="29">
+        <f t="shared" ref="E4:F7" ca="1" si="2">$B4*C4</f>
+        <v>96</v>
+      </c>
+      <c r="F4" s="36">
+        <f t="shared" ca="1" si="2"/>
+        <v>288</v>
+      </c>
+      <c r="G4" s="38">
+        <f ca="1">(E4+F4)/(E$8+F$8)</f>
+        <v>0.26175869120654399</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="24">
+        <f t="shared" ca="1" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="C5" s="31">
+        <f t="shared" ca="1" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="D5" s="28">
+        <f t="shared" ca="1" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E5" s="29">
+        <f t="shared" ca="1" si="2"/>
+        <v>130</v>
+      </c>
+      <c r="F5" s="35">
+        <f t="shared" ca="1" si="2"/>
+        <v>117</v>
+      </c>
+      <c r="G5" s="38">
+        <f t="shared" ref="G5:G7" ca="1" si="3">(E5+F5)/(E$8+F$8)</f>
+        <v>0.16837082481254259</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="39">
-        <f t="shared" ref="C4:D7" ca="1" si="1">RANDBETWEEN(2, 10)</f>
-        <v>10</v>
-      </c>
-      <c r="D4" s="33">
+      <c r="B6" s="24">
+        <f t="shared" ca="1" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="C6" s="26">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="D6" s="25">
+        <f t="shared" ca="1" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="E6" s="29">
+        <f t="shared" ca="1" si="2"/>
+        <v>64</v>
+      </c>
+      <c r="F6" s="35">
+        <f t="shared" ca="1" si="2"/>
+        <v>192</v>
+      </c>
+      <c r="G6" s="38">
+        <f t="shared" ca="1" si="3"/>
+        <v>0.17450579413769599</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="33">
+        <f t="shared" ca="1" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="C7" s="32">
         <f t="shared" ca="1" si="1"/>
         <v>5</v>
       </c>
-      <c r="E4" s="37">
-        <f t="shared" ref="E4:F7" ca="1" si="2">$B4*C4</f>
-        <v>400</v>
-      </c>
-      <c r="F4" s="45">
-        <f t="shared" ca="1" si="2"/>
-        <v>200</v>
-      </c>
-      <c r="G4" s="47">
-        <f ca="1">(E4+F4)/(E$8+F$8)</f>
-        <v>0.27051397655545534</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="32">
-        <f t="shared" ca="1" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="C5" s="39">
-        <f t="shared" ca="1" si="1"/>
-        <v>8</v>
-      </c>
-      <c r="D5" s="36">
+      <c r="D7" s="27">
         <f t="shared" ca="1" si="1"/>
         <v>3</v>
       </c>
-      <c r="E5" s="37">
+      <c r="E7" s="29">
         <f t="shared" ca="1" si="2"/>
-        <v>192</v>
-      </c>
-      <c r="F5" s="44">
+        <v>225</v>
+      </c>
+      <c r="F7" s="35">
         <f t="shared" ca="1" si="2"/>
-        <v>72</v>
-      </c>
-      <c r="G5" s="47">
-        <f t="shared" ref="G5:G7" ca="1" si="3">(E5+F5)/(E$8+F$8)</f>
-        <v>0.11902614968440037</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="31" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="32">
-        <f t="shared" ca="1" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="C6" s="34">
-        <f t="shared" ca="1" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="D6" s="33">
-        <f t="shared" ca="1" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="E6" s="37">
-        <f t="shared" ca="1" si="2"/>
-        <v>60</v>
-      </c>
-      <c r="F6" s="44">
-        <f t="shared" ca="1" si="2"/>
-        <v>60</v>
-      </c>
-      <c r="G6" s="47">
+        <v>135</v>
+      </c>
+      <c r="G7" s="38">
         <f t="shared" ca="1" si="3"/>
-        <v>5.4102795311091072E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="31" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="41">
-        <f t="shared" ca="1" si="0"/>
-        <v>44</v>
-      </c>
-      <c r="C7" s="40">
-        <f t="shared" ca="1" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="D7" s="35">
-        <f t="shared" ca="1" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="E7" s="37">
-        <f t="shared" ca="1" si="2"/>
-        <v>220</v>
-      </c>
-      <c r="F7" s="44">
-        <f t="shared" ca="1" si="2"/>
-        <v>440</v>
-      </c>
-      <c r="G7" s="47">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.29756537421100088</v>
+        <v>0.24539877300613497</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="43"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="46">
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="37">
         <f ca="1">SUM(E3:E7)</f>
-        <v>1118</v>
-      </c>
-      <c r="F8" s="46">
+        <v>575</v>
+      </c>
+      <c r="F8" s="37">
         <f ca="1">SUM(F3:F7)</f>
-        <v>1100</v>
-      </c>
-      <c r="G8" s="43"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C9" s="42"/>
+        <v>892</v>
+      </c>
+      <c r="G8" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2085,215 +3778,215 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="48" t="s">
+      <c r="C1" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="49"/>
+      <c r="G1" s="64"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="51">
+      <c r="C2" s="41">
         <f ca="1">RANDBETWEEN(500, 1000)</f>
+        <v>892</v>
+      </c>
+      <c r="F2" s="45" t="s">
+        <v>48</v>
+      </c>
+      <c r="G2" s="46">
+        <f ca="1">SUMIF($A$2:$A$9, F2, $C$2:$C$9)</f>
+        <v>1533</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="53" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="49" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" s="44">
+        <f t="shared" ref="C3:C9" ca="1" si="0">RANDBETWEEN(500, 1000)</f>
+        <v>690</v>
+      </c>
+      <c r="F3" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" s="34">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F3)</f>
+        <v>598</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="52" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="44">
+        <f t="shared" ca="1" si="0"/>
+        <v>621</v>
+      </c>
+      <c r="F4" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" s="34">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F4)</f>
+        <v>935</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="53" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="49" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="44">
+        <f t="shared" ca="1" si="0"/>
+        <v>641</v>
+      </c>
+      <c r="F5" s="45" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="46">
+        <f ca="1">SUMIF($A$2:$A$9, F5, $C$2:$C$9)</f>
+        <v>1582</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="52" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="44">
+        <f t="shared" ca="1" si="0"/>
+        <v>598</v>
+      </c>
+      <c r="F6" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="34">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F6)</f>
+        <v>892</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="53" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="49" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="44">
+        <f t="shared" ca="1" si="0"/>
+        <v>935</v>
+      </c>
+      <c r="F7" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" s="34">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F7)</f>
+        <v>690</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="52" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="44">
+        <f t="shared" ca="1" si="0"/>
+        <v>898</v>
+      </c>
+      <c r="F8" s="45" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="46">
+        <f ca="1">SUMIF($A$2:$A$9, F8, $C$2:$C$9)</f>
+        <v>1262</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="54" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="42">
+        <f t="shared" ca="1" si="0"/>
         <v>811</v>
       </c>
-      <c r="F2" s="55" t="s">
-        <v>48</v>
-      </c>
-      <c r="G2" s="56">
-        <f ca="1">SUMIF($A$2:$A$9, F2, $C$2:$C$9)</f>
-        <v>1673</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="63" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="59" t="s">
+      <c r="F9" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="34">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F9)</f>
+        <v>621</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F10" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="54">
-        <f t="shared" ref="C3:C9" ca="1" si="0">RANDBETWEEN(500, 1000)</f>
-        <v>688</v>
-      </c>
-      <c r="F3" s="43" t="s">
+      <c r="G10" s="34">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F10)</f>
+        <v>641</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F11" s="45" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="46">
+        <f ca="1">SUMIF($A$2:$A$9, F11, $C$2:$C$9)</f>
+        <v>1709</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F12" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="G3" s="43">
-        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F3)</f>
-        <v>721</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="62" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="58" t="s">
-        <v>50</v>
-      </c>
-      <c r="C4" s="54">
-        <f t="shared" ca="1" si="0"/>
-        <v>706</v>
-      </c>
-      <c r="F4" s="43" t="s">
+      <c r="G12" s="34">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F12)</f>
+        <v>898</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F13" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="G4" s="43">
-        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F4)</f>
-        <v>952</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="63" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="59" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="54">
-        <f t="shared" ca="1" si="0"/>
-        <v>680</v>
-      </c>
-      <c r="F5" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="G5" s="56">
-        <f ca="1">SUMIF($A$2:$A$9, F5, $C$2:$C$9)</f>
-        <v>1499</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="62" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="58" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6" s="54">
-        <f t="shared" ca="1" si="0"/>
-        <v>721</v>
-      </c>
-      <c r="F6" s="43" t="s">
-        <v>50</v>
-      </c>
-      <c r="G6" s="43">
-        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F6)</f>
+      <c r="G13" s="34">
+        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F13)</f>
         <v>811</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="63" t="s">
-        <v>48</v>
-      </c>
-      <c r="B7" s="59" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="54">
-        <f t="shared" ca="1" si="0"/>
-        <v>952</v>
-      </c>
-      <c r="F7" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="43">
-        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F7)</f>
-        <v>688</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="62" t="s">
-        <v>49</v>
-      </c>
-      <c r="B8" s="58" t="s">
-        <v>50</v>
-      </c>
-      <c r="C8" s="54">
-        <f t="shared" ca="1" si="0"/>
-        <v>646</v>
-      </c>
-      <c r="F8" s="55" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="56">
-        <f ca="1">SUMIF($A$2:$A$9, F8, $C$2:$C$9)</f>
-        <v>1386</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="64" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="52">
-        <f t="shared" ca="1" si="0"/>
-        <v>968</v>
-      </c>
-      <c r="F9" s="43" t="s">
-        <v>50</v>
-      </c>
-      <c r="G9" s="43">
-        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F9)</f>
-        <v>706</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F10" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="G10" s="43">
-        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F10)</f>
-        <v>680</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F11" s="55" t="s">
-        <v>49</v>
-      </c>
-      <c r="G11" s="56">
-        <f ca="1">SUMIF($A$2:$A$9, F11, $C$2:$C$9)</f>
-        <v>1614</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F12" s="43" t="s">
-        <v>50</v>
-      </c>
-      <c r="G12" s="43">
-        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F12)</f>
-        <v>646</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F13" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="G13" s="43">
-        <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F13)</f>
-        <v>968</v>
-      </c>
-    </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F14" s="50" t="s">
+      <c r="F14" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="G14" s="53">
+      <c r="G14" s="43">
         <f ca="1">SUM(G2,G5,G8,G11)</f>
-        <v>6172</v>
+        <v>6086</v>
       </c>
     </row>
   </sheetData>
@@ -2306,187 +3999,437 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22AB70FF-96FA-4025-A517-8BDE3ECE5EBF}">
-  <dimension ref="B1:F9"/>
+  <dimension ref="B1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" style="65" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" style="65" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" style="65" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.28515625" style="65" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" style="65" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" style="55" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" style="55" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="55" customWidth="1"/>
+    <col min="5" max="5" width="28.5703125" style="55" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" style="55" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="69" t="s">
+      <c r="C1" s="66" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="69" t="s">
+      <c r="D1" s="66" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="70" t="s">
+      <c r="E1" s="67" t="s">
         <v>56</v>
       </c>
       <c r="F1" s="68" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="65" t="s">
-        <v>58</v>
-      </c>
-      <c r="C2" s="65" t="s">
+    <row r="2" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="69" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="69" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="69" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" s="70">
+        <v>60000</v>
+      </c>
+      <c r="F2" s="71">
+        <f>DATE(2026, 10, 5)</f>
+        <v>46300</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="69" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="69" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="69" t="s">
+        <v>68</v>
+      </c>
+      <c r="E3" s="70">
+        <v>50000</v>
+      </c>
+      <c r="F3" s="71">
+        <f>DATE(2026, 4, 7)</f>
+        <v>46119</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="69" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="69" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" s="69" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="70">
+        <v>25000</v>
+      </c>
+      <c r="F4" s="71">
+        <f>DATE(2026, 8, 7)</f>
+        <v>46241</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="69" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="69" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="69" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="70">
+        <v>15000</v>
+      </c>
+      <c r="F5" s="71">
+        <f>DATE(2026, 5, 8)</f>
+        <v>46150</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="69" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="69" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="65" t="s">
-        <v>66</v>
-      </c>
-      <c r="E2" s="66">
-        <f ca="1">RANDBETWEEN(5000, 80000)</f>
-        <v>21206</v>
-      </c>
-      <c r="F2" s="67">
+      <c r="E6" s="70">
+        <v>10000</v>
+      </c>
+      <c r="F6" s="71">
+        <f>DATE(2026, 9, 7)</f>
+        <v>46272</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="69" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="69" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" s="69" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="70">
+        <v>7500</v>
+      </c>
+      <c r="F7" s="71">
         <f>DATE(2026, 5, 7)</f>
         <v>46149</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="65" t="s">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="69" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="69" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="69" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="70">
+        <v>7000</v>
+      </c>
+      <c r="F8" s="71">
+        <f>DATE(2026, 5, 7)</f>
+        <v>46149</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="72" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="65" t="s">
+      <c r="C9" s="72" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="65" t="s">
+      <c r="D9" s="72" t="s">
         <v>67</v>
       </c>
-      <c r="E3" s="66">
-        <f t="shared" ref="E3:E9" ca="1" si="0">RANDBETWEEN(5000, 80000)</f>
-        <v>14031</v>
-      </c>
-      <c r="F3" s="67">
-        <f>DATE(2026, 6, 7)</f>
-        <v>46180</v>
-      </c>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="65" t="s">
-        <v>60</v>
-      </c>
-      <c r="C4" s="65" t="s">
-        <v>68</v>
-      </c>
-      <c r="D4" s="65" t="s">
-        <v>68</v>
-      </c>
-      <c r="E4" s="66">
-        <f t="shared" ca="1" si="0"/>
-        <v>14215</v>
-      </c>
-      <c r="F4" s="67">
-        <f>DATE(2026, 7, 7)</f>
-        <v>46210</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="65" t="s">
-        <v>61</v>
-      </c>
-      <c r="C5" s="65" t="s">
-        <v>69</v>
-      </c>
-      <c r="D5" s="65" t="s">
-        <v>69</v>
-      </c>
-      <c r="E5" s="66">
-        <f t="shared" ca="1" si="0"/>
-        <v>44607</v>
-      </c>
-      <c r="F5" s="67">
-        <f>DATE(2026, 8, 7)</f>
-        <v>46241</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="65" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" s="65" t="s">
-        <v>70</v>
-      </c>
-      <c r="D6" s="65" t="s">
-        <v>70</v>
-      </c>
-      <c r="E6" s="66">
-        <f t="shared" ca="1" si="0"/>
-        <v>64020</v>
-      </c>
-      <c r="F6" s="67">
-        <f>DATE(2026, 9, 7)</f>
-        <v>46272</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="65" t="s">
-        <v>63</v>
-      </c>
-      <c r="C7" s="65" t="s">
-        <v>71</v>
-      </c>
-      <c r="D7" s="65" t="s">
-        <v>71</v>
-      </c>
-      <c r="E7" s="66">
-        <f t="shared" ca="1" si="0"/>
-        <v>8305</v>
-      </c>
-      <c r="F7" s="67">
-        <f>DATE(2026, 10, 7)</f>
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="65" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="65" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="65" t="s">
-        <v>72</v>
-      </c>
-      <c r="E8" s="66">
-        <f t="shared" ca="1" si="0"/>
-        <v>8319</v>
-      </c>
-      <c r="F8" s="67">
-        <f>DATE(2026, 11, 7)</f>
-        <v>46333</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="65" t="s">
-        <v>65</v>
-      </c>
-      <c r="C9" s="65" t="s">
-        <v>73</v>
-      </c>
-      <c r="D9" s="65" t="s">
-        <v>73</v>
-      </c>
-      <c r="E9" s="66">
-        <f t="shared" ca="1" si="0"/>
-        <v>70353</v>
-      </c>
-      <c r="F9" s="67">
-        <f>DATE(2026, 12, 7)</f>
-        <v>46363</v>
+      <c r="E9" s="73">
+        <v>6000</v>
+      </c>
+      <c r="F9" s="74">
+        <f>DATE(2026, 6, 6)</f>
+        <v>46179</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C12" s="75" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="75"/>
+      <c r="E12" s="76">
+        <f>SUM(JLoka_Investors[INVESTMENT AMOUNT (USD)])</f>
+        <v>180500</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:F9">
+    <sortCondition descending="1" ref="E2:E9"/>
+  </sortState>
+  <mergeCells count="1">
+    <mergeCell ref="C12:D12"/>
+  </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{3A4CF648-6AED-40f4-86FF-DC5316D8AED3}">
+      <x14:slicerList xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
+        <x14:slicer r:id="rId3"/>
+      </x14:slicerList>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DED3323-DAD4-4089-9A46-7712A3CF5F64}">
+  <dimension ref="B2:F14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B2" s="78" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="77"/>
+    </row>
+    <row r="3" spans="2:6" s="77" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="77" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="77" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="77" t="s">
+        <v>78</v>
+      </c>
+      <c r="E3" s="77" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>2011</v>
+      </c>
+      <c r="C4" s="3">
+        <f ca="1">RAND()</f>
+        <v>0.74632334827253011</v>
+      </c>
+      <c r="D4" s="3">
+        <f t="shared" ref="D4:E4" ca="1" si="0">RAND()</f>
+        <v>7.6764236190715374E-2</v>
+      </c>
+      <c r="E4" s="3">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.59766622878496245</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>2012</v>
+      </c>
+      <c r="C5" s="3">
+        <f t="shared" ref="C5:E14" ca="1" si="1">RAND()</f>
+        <v>0.96726538064451084</v>
+      </c>
+      <c r="D5" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>5.4354528886120357E-2</v>
+      </c>
+      <c r="E5" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.35034220588725351</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>2013</v>
+      </c>
+      <c r="C6" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.34234357821502415</v>
+      </c>
+      <c r="D6" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.28344606593773036</v>
+      </c>
+      <c r="E6" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.69553741865844598</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>2014</v>
+      </c>
+      <c r="C7" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.6802225754616299</v>
+      </c>
+      <c r="D7" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.71322647348581636</v>
+      </c>
+      <c r="E7" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.58331324969536502</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>2015</v>
+      </c>
+      <c r="C8" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.41154429073134569</v>
+      </c>
+      <c r="D8" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.24424704666357588</v>
+      </c>
+      <c r="E8" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>4.5648847882053256E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9">
+        <v>2016</v>
+      </c>
+      <c r="C9" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>2.8166285419759518E-3</v>
+      </c>
+      <c r="D9" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>9.6777844968651827E-2</v>
+      </c>
+      <c r="E9" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.70430520884159553</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>2017</v>
+      </c>
+      <c r="C10" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.55602648328598325</v>
+      </c>
+      <c r="D10" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.52020423431596585</v>
+      </c>
+      <c r="E10" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.34173611134409643</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>2018</v>
+      </c>
+      <c r="C11" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.72204098578482745</v>
+      </c>
+      <c r="D11" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.32085133206821126</v>
+      </c>
+      <c r="E11" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.38026533146699537</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <v>2019</v>
+      </c>
+      <c r="C12" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.75989775807371251</v>
+      </c>
+      <c r="D12" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.47604524511131241</v>
+      </c>
+      <c r="E12" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.61216195487650615</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13">
+        <v>2020</v>
+      </c>
+      <c r="C13" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.36214243666635559</v>
+      </c>
+      <c r="D13" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.96824967018629216</v>
+      </c>
+      <c r="E13" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.94629380652869344</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14">
+        <v>2021</v>
+      </c>
+      <c r="C14" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>8.0557715692428644E-3</v>
+      </c>
+      <c r="D14" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.99040654877882894</v>
+      </c>
+      <c r="E14" s="3">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.8497834350972423</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adding Finance with Excel Sample
</commit_message>
<xml_diff>
--- a/Excel-Finance/JLoka-Finance-01.xlsx
+++ b/Excel-Finance/JLoka-Finance-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\books-and-tutorials\Finance-Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F41F8F-04F6-40F5-BA6F-2BFC3A455D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F6522C-427F-48A1-9567-6B6BBB9E8212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,9 @@
     <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
     <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
     <sheet name="Sheet8" sheetId="8" r:id="rId8"/>
+    <sheet name="Sheet9" sheetId="9" r:id="rId9"/>
+    <sheet name="Sheet10" sheetId="10" r:id="rId10"/>
+    <sheet name="Sheet11" sheetId="11" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet7!$B$1:$F$9</definedName>
@@ -34,8 +37,8 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicerCache r:id="rId9"/>
-        <x14:slicerCache r:id="rId10"/>
+        <x14:slicerCache r:id="rId12"/>
+        <x14:slicerCache r:id="rId13"/>
       </x15:slicerCaches>
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -55,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="122">
   <si>
     <t>Sunday</t>
   </si>
@@ -295,16 +298,143 @@
   </si>
   <si>
     <t>Jloka-03</t>
+  </si>
+  <si>
+    <t>Investment Type</t>
+  </si>
+  <si>
+    <t>Portfolio Allocation</t>
+  </si>
+  <si>
+    <t>Stocks</t>
+  </si>
+  <si>
+    <t>Bonds</t>
+  </si>
+  <si>
+    <t>Real Estate</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>Applicant</t>
+  </si>
+  <si>
+    <t>Credit Score</t>
+  </si>
+  <si>
+    <t>Loan Amount</t>
+  </si>
+  <si>
+    <t>Employement Status</t>
+  </si>
+  <si>
+    <t>Good Credit?</t>
+  </si>
+  <si>
+    <t>Approved or Denied?</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>Full-Time</t>
+  </si>
+  <si>
+    <t>Part-Time</t>
+  </si>
+  <si>
+    <t>UnEmployment</t>
+  </si>
+  <si>
+    <t>Ticker</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Dividend</t>
+  </si>
+  <si>
+    <t>Jloka-04</t>
+  </si>
+  <si>
+    <t>Jloka-05</t>
+  </si>
+  <si>
+    <t>Jloka-06</t>
+  </si>
+  <si>
+    <t>Jloka-07</t>
+  </si>
+  <si>
+    <t>Jloka-08</t>
+  </si>
+  <si>
+    <t>Jloka-09</t>
+  </si>
+  <si>
+    <t>Jloka-10</t>
+  </si>
+  <si>
+    <t>Jloka-100</t>
+  </si>
+  <si>
+    <t>Jloka-101</t>
+  </si>
+  <si>
+    <t>Jloka-102</t>
+  </si>
+  <si>
+    <t>Jloka-103</t>
+  </si>
+  <si>
+    <t>Jloka-104</t>
+  </si>
+  <si>
+    <t>Jloka-105</t>
+  </si>
+  <si>
+    <t>Jloka-106</t>
+  </si>
+  <si>
+    <t>Jloka-107</t>
+  </si>
+  <si>
+    <t>Jloka-108</t>
+  </si>
+  <si>
+    <t>Jloka-109</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -765,7 +895,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -834,6 +964,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -861,46 +1031,13 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -909,9 +1046,25 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="23">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -930,6 +1083,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="166" formatCode="0.0%"/>
     </dxf>
     <dxf>
       <font>
@@ -989,10 +1143,28 @@
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="166" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -1110,6 +1282,48 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1149,19 +1363,13 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1320" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="95000"/>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
-                    <a:prstClr val="black">
-                      <a:alpha val="40000"/>
-                    </a:prstClr>
-                  </a:outerShdw>
-                </a:effectLst>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
@@ -1169,8 +1377,13 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Stock Returns</a:t>
+              <a:t>JLoka</a:t>
             </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Sock Returns</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -1187,19 +1400,13 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1320" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
+            <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="95000"/>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
-                  <a:prstClr val="black">
-                    <a:alpha val="40000"/>
-                  </a:prstClr>
-                </a:outerShdw>
-              </a:effectLst>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
@@ -1219,60 +1426,111 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:spPr>
-            <a:ln w="34925" cap="rnd">
+            <a:ln w="28575" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
+            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="l"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet8!$B$4:$B$14</c:f>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Sheet8!$B$4:$B$14</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Sheet8!$B$6:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>2011</c:v>
+                  <c:v>2013</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2012</c:v>
+                  <c:v>2014</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2013</c:v>
+                  <c:v>2015</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2014</c:v>
+                  <c:v>2016</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2015</c:v>
+                  <c:v>2017</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2016</c:v>
+                  <c:v>2018</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2017</c:v>
+                  <c:v>2019</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2018</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2019</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>2020</c:v>
-                </c:pt>
-                <c:pt idx="10">
                   <c:v>2021</c:v>
                 </c:pt>
               </c:numCache>
@@ -1280,42 +1538,43 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet8!$C$4:$C$14</c:f>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Sheet8!$C$4:$C$14</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Sheet8!$C$6:$C$14</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.74632334827253011</c:v>
+                  <c:v>0.92177328897518906</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.96726538064451084</c:v>
+                  <c:v>6.8127943760001086E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.34234357821502415</c:v>
+                  <c:v>0.36546159306277792</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.6802225754616299</c:v>
+                  <c:v>7.0132702277079795E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.41154429073134569</c:v>
+                  <c:v>0.29363415525332215</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.8166285419759518E-3</c:v>
+                  <c:v>0.57614710490615306</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.55602648328598325</c:v>
+                  <c:v>0.42653486070031332</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.72204098578482745</c:v>
+                  <c:v>0.27532486384594812</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.75989775807371251</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.36214243666635559</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>8.0557715692428644E-3</c:v>
+                  <c:v>0.39228657162766789</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1323,7 +1582,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9F87-4B16-9178-53052F6E00C5}"/>
+              <c16:uniqueId val="{00000000-DCD0-4F92-BB1E-6308041B97FE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1331,60 +1590,111 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:spPr>
-            <a:ln w="34925" cap="rnd">
+            <a:ln w="28575" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
+            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="l"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet8!$B$4:$B$14</c:f>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Sheet8!$B$4:$B$14</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Sheet8!$B$6:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>2011</c:v>
+                  <c:v>2013</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2012</c:v>
+                  <c:v>2014</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2013</c:v>
+                  <c:v>2015</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2014</c:v>
+                  <c:v>2016</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2015</c:v>
+                  <c:v>2017</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2016</c:v>
+                  <c:v>2018</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2017</c:v>
+                  <c:v>2019</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2018</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2019</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>2020</c:v>
-                </c:pt>
-                <c:pt idx="10">
                   <c:v>2021</c:v>
                 </c:pt>
               </c:numCache>
@@ -1392,42 +1702,43 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet8!$D$4:$D$14</c:f>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Sheet8!$D$4:$D$14</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Sheet8!$D$6:$D$14</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>7.6764236190715374E-2</c:v>
+                  <c:v>0.62960068734179109</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.4354528886120357E-2</c:v>
+                  <c:v>0.91148131598852689</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.28344606593773036</c:v>
+                  <c:v>0.49768864602230933</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.71322647348581636</c:v>
+                  <c:v>0.39161580424131404</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.24424704666357588</c:v>
+                  <c:v>3.4430219338273838E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>9.6777844968651827E-2</c:v>
+                  <c:v>0.88951744204066985</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.52020423431596585</c:v>
+                  <c:v>0.21054797943785342</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.32085133206821126</c:v>
+                  <c:v>0.29914873161213729</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.47604524511131241</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.96824967018629216</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.99040654877882894</c:v>
+                  <c:v>0.72402950173284431</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1435,7 +1746,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-9F87-4B16-9178-53052F6E00C5}"/>
+              <c16:uniqueId val="{00000001-DCD0-4F92-BB1E-6308041B97FE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1443,60 +1754,111 @@
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:spPr>
-            <a:ln w="34925" cap="rnd">
+            <a:ln w="28575" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent3"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
+            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="l"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet8!$B$4:$B$14</c:f>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Sheet8!$B$4:$B$14</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Sheet8!$B$6:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>2011</c:v>
+                  <c:v>2013</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2012</c:v>
+                  <c:v>2014</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2013</c:v>
+                  <c:v>2015</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2014</c:v>
+                  <c:v>2016</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2015</c:v>
+                  <c:v>2017</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2016</c:v>
+                  <c:v>2018</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2017</c:v>
+                  <c:v>2019</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2018</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2019</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>2020</c:v>
-                </c:pt>
-                <c:pt idx="10">
                   <c:v>2021</c:v>
                 </c:pt>
               </c:numCache>
@@ -1504,42 +1866,43 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet8!$E$4:$E$14</c:f>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Sheet8!$E$4:$E$14</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Sheet8!$E$6:$E$14</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.59766622878496245</c:v>
+                  <c:v>0.47613209032723569</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.35034220588725351</c:v>
+                  <c:v>0.33943465465660472</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.69553741865844598</c:v>
+                  <c:v>0.56689538950625051</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.58331324969536502</c:v>
+                  <c:v>0.70946690247282718</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.5648847882053256E-2</c:v>
+                  <c:v>0.48517707387830089</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.70430520884159553</c:v>
+                  <c:v>0.34191490610491293</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.34173611134409643</c:v>
+                  <c:v>0.75340815882757395</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.38026533146699537</c:v>
+                  <c:v>0.73473476496323886</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.61216195487650615</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.94629380652869344</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.8497834350972423</c:v>
+                  <c:v>6.5175240099631937E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1547,24 +1910,25 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-9F87-4B16-9178-53052F6E00C5}"/>
+              <c16:uniqueId val="{00000002-DCD0-4F92-BB1E-6308041B97FE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:dLblPos val="l"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
+          <c:showVal val="1"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="1734618992"/>
-        <c:axId val="1734630512"/>
+        <c:axId val="1180860607"/>
+        <c:axId val="1180858207"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1734618992"/>
+        <c:axId val="1180860607"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1578,9 +1942,9 @@
           <a:noFill/>
           <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="lt1">
-                <a:lumMod val="95000"/>
-                <a:alpha val="10000"/>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:round/>
@@ -1592,10 +1956,11 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="85000"/>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -1606,7 +1971,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1734630512"/>
+        <c:crossAx val="1180858207"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1614,7 +1979,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1734630512"/>
+        <c:axId val="1180858207"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1624,9 +1989,9 @@
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="95000"/>
-                  <a:alpha val="10000"/>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:round/>
@@ -1650,10 +2015,11 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="85000"/>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -1664,10 +2030,49 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1734618992"/>
+        <c:crossAx val="1180860607"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:dTable>
+        <c:showHorzBorder val="1"/>
+        <c:showVertBorder val="1"/>
+        <c:showOutline val="1"/>
+        <c:showKeys val="0"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr rtl="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+      </c:dTable>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -1691,10 +2096,11 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="85000"/>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
@@ -1711,28 +2117,17 @@
     <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
-    <a:gradFill flip="none" rotWithShape="1">
-      <a:gsLst>
-        <a:gs pos="0">
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:gs>
-        <a:gs pos="100000">
-          <a:schemeClr val="dk1">
-            <a:lumMod val="85000"/>
-            <a:lumOff val="15000"/>
-          </a:schemeClr>
-        </a:gs>
-      </a:gsLst>
-      <a:path path="circle">
-        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-      </a:path>
-      <a:tileRect/>
-    </a:gradFill>
-    <a:ln>
-      <a:noFill/>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
     </a:ln>
     <a:effectLst/>
   </c:spPr>
@@ -1741,7 +2136,475 @@
     <a:lstStyle/>
     <a:p>
       <a:pPr>
-        <a:defRPr sz="1100" b="1"/>
+        <a:defRPr b="1"/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1440" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx2"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>The Potfolio Allocation</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1440" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx2"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:view3D>
+      <c:rotX val="30"/>
+      <c:rotY val="0"/>
+      <c:depthPercent val="100"/>
+      <c:rAngAx val="0"/>
+    </c:view3D>
+    <c:floor>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:floor>
+    <c:sideWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:sideWall>
+    <c:backWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:backWall>
+    <c:plotArea>
+      <c:layout/>
+      <c:pie3DChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:gradFill rotWithShape="1">
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent1">
+                      <a:satMod val="103000"/>
+                      <a:lumMod val="102000"/>
+                      <a:tint val="94000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="50000">
+                    <a:schemeClr val="accent1">
+                      <a:satMod val="110000"/>
+                      <a:lumMod val="100000"/>
+                      <a:shade val="100000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="99000"/>
+                      <a:satMod val="120000"/>
+                      <a:shade val="78000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000" scaled="0"/>
+              </a:gradFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-45A3-40A4-989A-7A690D2C05E7}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:gradFill rotWithShape="1">
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent2">
+                      <a:satMod val="103000"/>
+                      <a:lumMod val="102000"/>
+                      <a:tint val="94000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="50000">
+                    <a:schemeClr val="accent2">
+                      <a:satMod val="110000"/>
+                      <a:lumMod val="100000"/>
+                      <a:shade val="100000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent2">
+                      <a:lumMod val="99000"/>
+                      <a:satMod val="120000"/>
+                      <a:shade val="78000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000" scaled="0"/>
+              </a:gradFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-45A3-40A4-989A-7A690D2C05E7}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:gradFill rotWithShape="1">
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent3">
+                      <a:satMod val="103000"/>
+                      <a:lumMod val="102000"/>
+                      <a:tint val="94000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="50000">
+                    <a:schemeClr val="accent3">
+                      <a:satMod val="110000"/>
+                      <a:lumMod val="100000"/>
+                      <a:shade val="100000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent3">
+                      <a:lumMod val="99000"/>
+                      <a:satMod val="120000"/>
+                      <a:shade val="78000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000" scaled="0"/>
+              </a:gradFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-45A3-40A4-989A-7A690D2C05E7}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:gradFill rotWithShape="1">
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent4">
+                      <a:satMod val="103000"/>
+                      <a:lumMod val="102000"/>
+                      <a:tint val="94000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="50000">
+                    <a:schemeClr val="accent4">
+                      <a:satMod val="110000"/>
+                      <a:lumMod val="100000"/>
+                      <a:shade val="100000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent4">
+                      <a:lumMod val="99000"/>
+                      <a:satMod val="120000"/>
+                      <a:shade val="78000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000" scaled="0"/>
+              </a:gradFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-45A3-40A4-989A-7A690D2C05E7}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx2"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="bestFit"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="tx2">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet9!$B$3:$B$6</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Stocks</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Bonds</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Real Estate</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Cash</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet9!$C$3:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.60699999999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.29299999999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.5000000000000002E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.5000000000000003E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-00FD-4EB6-A61E-FA78A920F0AB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="bestFit"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+      </c:pie3DChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx2"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx2">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="1200" b="1"/>
       </a:pPr>
       <a:endParaRPr lang="en-US"/>
     </a:p>
@@ -1794,34 +2657,76 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="233">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
+    <cs:defRPr sz="1000" kern="1200"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="10000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1829,34 +2734,26 @@
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:categoryAxis>
-  <cs:chartArea>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:gradFill flip="none" rotWithShape="1">
-        <a:gsLst>
-          <a:gs pos="0">
-            <a:schemeClr val="dk1">
-              <a:lumMod val="65000"/>
-              <a:lumOff val="35000"/>
-            </a:schemeClr>
-          </a:gs>
-          <a:gs pos="100000">
-            <a:schemeClr val="dk1">
-              <a:lumMod val="85000"/>
-              <a:lumOff val="15000"/>
-            </a:schemeClr>
-          </a:gs>
-        </a:gsLst>
-        <a:path path="circle">
-          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-        </a:path>
-        <a:tileRect/>
-      </a:gradFill>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="1000" kern="1200"/>
   </cs:chartArea>
@@ -1865,8 +2762,9 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -1885,6 +2783,14 @@
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -1893,35 +2799,45 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="3">
+    <cs:fillRef idx="1">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="3"/>
+    <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="3">
+    <cs:fillRef idx="1">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="3"/>
+    <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="3"/>
-    <cs:effectRef idx="3"/>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="34925" cap="rnd">
+      <a:ln w="28575" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -1933,29 +2849,31 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="3">
+    <cs:fillRef idx="1">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="3"/>
+    <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="3"/>
-    <cs:effectRef idx="3"/>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
@@ -1973,18 +2891,21 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
@@ -1994,20 +2915,20 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
         </a:schemeClr>
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -2021,14 +2942,14 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:prstDash val="dash"/>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dropLine>
@@ -2042,8 +2963,9 @@
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2057,6 +2979,12 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
   </cs:floor>
   <cs:gridlineMajor>
     <cs:lnRef idx="0"/>
@@ -2068,9 +2996,9 @@
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="10000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2085,13 +3013,14 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="5000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:gridlineMinor>
@@ -2103,14 +3032,14 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:prstDash val="dash"/>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:hiLoLine>
@@ -2122,13 +3051,14 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:leaderLine>
@@ -2137,13 +3067,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:legend>
-  <cs:plotArea>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
@@ -2151,7 +3082,7 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
   </cs:plotArea>
-  <cs:plotArea3D>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
@@ -2164,21 +3095,11 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:seriesAxis>
   <cs:seriesLine>
@@ -2186,14 +3107,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2205,19 +3126,12 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="95000"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
-      <a:effectLst>
-        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
-          <a:prstClr val="black">
-            <a:alpha val="40000"/>
-          </a:prstClr>
-        </a:outerShdw>
-      </a:effectLst>
-    </cs:defRPr>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
   </cs:title>
   <cs:trendline>
     <cs:lnRef idx="0">
@@ -2233,6 +3147,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:prstDash val="sysDot"/>
       </a:ln>
     </cs:spPr>
   </cs:trendline>
@@ -2241,8 +3156,9 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -2252,7 +3168,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -2260,9 +3176,9 @@
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -2273,8 +3189,9 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -2285,6 +3202,480 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="266">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk2">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700">
+        <a:solidFill>
+          <a:schemeClr val="lt2"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
@@ -2305,8 +3696,8 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer" Requires="sle15">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+      <mc:Choice Requires="sle15">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="2" name="COMPANY_NAME">
@@ -2329,7 +3720,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -2383,8 +3774,8 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer" Requires="sle15">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+      <mc:Choice Requires="sle15">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="3" name="INVESTMENT AMOUNT (USD)">
@@ -2407,7 +3798,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -2455,23 +3846,64 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>352425</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>4762</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>190499</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>185736</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>85725</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>447674</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>123824</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8BA38FCA-E474-5F44-D2BD-43AF24612BA4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>14287</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D179C9A-3D96-A297-DF2A-3741166D9F0E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{813F01E7-24A8-C626-808C-37CA7D764BE3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2520,7 +3952,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{385DC015-9960-47FA-A637-6B66C3CB4FFA}" name="JLoka_Investors" displayName="JLoka_Investors" ref="B1:F9" totalsRowShown="0" dataDxfId="5" tableBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{385DC015-9960-47FA-A637-6B66C3CB4FFA}" name="JLoka_Investors" displayName="JLoka_Investors" ref="B1:F9" totalsRowShown="0" dataDxfId="15" tableBorderDxfId="14">
   <autoFilter ref="B1:F9" xr:uid="{22AB70FF-96FA-4025-A517-8BDE3ECE5EBF}">
     <filterColumn colId="2">
       <filters>
@@ -2529,32 +3961,62 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{0BE1A407-37E2-45E1-A4B9-6EE27C852CA8}" name="INVESTOR_ID" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{F40E02B0-B4B8-4130-A683-00045FEF2BC6}" name="INVESTOR_NAME" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{EB541472-54EA-4246-959A-8F16F8FDA58F}" name="COMPANY_NAME" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{B149ED9E-81EF-4313-90DA-EDCF3ACBE03C}" name="INVESTMENT AMOUNT (USD)" dataDxfId="7" dataCellStyle="Currency"/>
-    <tableColumn id="5" xr3:uid="{5C700949-A13F-423E-81D1-C89753142DF7}" name="INVESTMENT_DATE" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{0BE1A407-37E2-45E1-A4B9-6EE27C852CA8}" name="INVESTOR_ID" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{F40E02B0-B4B8-4130-A683-00045FEF2BC6}" name="INVESTOR_NAME" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{EB541472-54EA-4246-959A-8F16F8FDA58F}" name="COMPANY_NAME" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{B149ED9E-81EF-4313-90DA-EDCF3ACBE03C}" name="INVESTMENT AMOUNT (USD)" dataDxfId="10" dataCellStyle="Currency"/>
+    <tableColumn id="5" xr3:uid="{5C700949-A13F-423E-81D1-C89753142DF7}" name="INVESTMENT_DATE" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E0111534-CC78-4AAC-9FB0-08AB9DCECE24}" name="Table4" displayName="Table4" ref="B3:E14" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" dataCellStyle="Percent">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E0111534-CC78-4AAC-9FB0-08AB9DCECE24}" name="Table4" displayName="Table4" ref="B3:E14" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7" dataCellStyle="Percent">
   <autoFilter ref="B3:E14" xr:uid="{E0111534-CC78-4AAC-9FB0-08AB9DCECE24}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{B5AEA49B-906B-4BA3-9E02-DF265E516312}" name="Year"/>
-    <tableColumn id="2" xr3:uid="{8C94788E-9FB3-46B0-A805-B97EFDDC36C5}" name="Jloka-01" dataDxfId="4" dataCellStyle="Percent">
+    <tableColumn id="2" xr3:uid="{8C94788E-9FB3-46B0-A805-B97EFDDC36C5}" name="Jloka-01" dataDxfId="6" dataCellStyle="Percent">
       <calculatedColumnFormula>RAND()</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A2693482-C7C8-4B05-9865-B12ABE5CC110}" name="Jloka-02" dataDxfId="3" dataCellStyle="Percent">
+    <tableColumn id="3" xr3:uid="{A2693482-C7C8-4B05-9865-B12ABE5CC110}" name="Jloka-02" dataDxfId="5" dataCellStyle="Percent">
       <calculatedColumnFormula>RAND()</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8F26A52C-2531-497C-A839-2A770D581E4E}" name="Jloka-03" dataDxfId="2" dataCellStyle="Percent">
+    <tableColumn id="4" xr3:uid="{8F26A52C-2531-497C-A839-2A770D581E4E}" name="Jloka-03" dataDxfId="4" dataCellStyle="Percent">
       <calculatedColumnFormula>RAND()</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{80A2B397-4223-4F15-9DB4-892BEE67AC07}" name="Table3" displayName="Table3" ref="B2:C6" totalsRowShown="0">
+  <autoFilter ref="B2:C6" xr:uid="{80A2B397-4223-4F15-9DB4-892BEE67AC07}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{C09EC9D1-D203-4F94-BBB0-27B52BD67348}" name="Investment Type"/>
+    <tableColumn id="2" xr3:uid="{DDA73600-5426-4CA3-8EA1-3D48A09909F0}" name="Portfolio Allocation" dataDxfId="3" dataCellStyle="Percent"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{26F768BE-F4AC-48CD-9271-53238CC90A9E}" name="Table5" displayName="Table5" ref="B2:G8" totalsRowShown="0" headerRowDxfId="22">
+  <autoFilter ref="B2:G8" xr:uid="{26F768BE-F4AC-48CD-9271-53238CC90A9E}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{CD0DE5D2-C8ED-45CF-8F5D-E6E88682B06A}" name="Applicant" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{89F30673-4126-482B-AFC9-E6FAD8DBE3F4}" name="Credit Score" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{4BC38630-914F-4BE8-9B0A-961F3FF855C4}" name="Loan Amount" dataDxfId="19" dataCellStyle="Currency"/>
+    <tableColumn id="4" xr3:uid="{7CE22975-ED55-49DD-B302-D5C876BF8196}" name="Employement Status" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{BD342C3D-5A81-4372-A781-AB1A62E26D7B}" name="Good Credit?" dataDxfId="17">
+      <calculatedColumnFormula>IF(Table5[[#This Row],[Credit Score]]&gt;700, "Yes", "No")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{14D8C1DF-DE7F-494A-8E09-15D4A0C38048}" name="Approved or Denied?" dataDxfId="16">
+      <calculatedColumnFormula>IF(OR(Table5[[#This Row],[Good Credit?]]="Yes", Table5[[#This Row],[Employement Status]]="Full-Time"), "Approved", IF(AND(C3&gt;650, Table5[[#This Row],[Loan Amount]]&lt;12000), "Approved", "Denied"))</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -2912,6 +4374,384 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A9EEF3-DE7A-4CAA-BA1C-C8A88C9A4643}">
+  <dimension ref="B2:G8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="4" width="17.140625" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="17.140625" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B2" s="67" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" s="67" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2" s="67" t="s">
+        <v>88</v>
+      </c>
+      <c r="E2" s="67" t="s">
+        <v>89</v>
+      </c>
+      <c r="F2" s="67" t="s">
+        <v>90</v>
+      </c>
+      <c r="G2" s="67" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="67" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" s="67">
+        <v>720</v>
+      </c>
+      <c r="D3" s="69">
+        <v>20000</v>
+      </c>
+      <c r="E3" s="67" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" t="str">
+        <f>IF(Table5[[#This Row],[Credit Score]]&gt;700, "Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="G3" s="67" t="str">
+        <f>IF(OR(Table5[[#This Row],[Good Credit?]]="Yes", Table5[[#This Row],[Employement Status]]="Full-Time"), "Approved", IF(AND(C3&gt;650, Table5[[#This Row],[Loan Amount]]&lt;12000), "Approved", "Denied"))</f>
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="67" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="67">
+        <v>680</v>
+      </c>
+      <c r="D4" s="69">
+        <v>15000</v>
+      </c>
+      <c r="E4" s="67" t="s">
+        <v>99</v>
+      </c>
+      <c r="F4" t="str">
+        <f>IF(Table5[[#This Row],[Credit Score]]&gt;700, "Yes", "No")</f>
+        <v>No</v>
+      </c>
+      <c r="G4" s="67" t="str">
+        <f>IF(OR(Table5[[#This Row],[Good Credit?]]="Yes", Table5[[#This Row],[Employement Status]]="Full-Time"), "Approved", IF(AND(C4&gt;650, Table5[[#This Row],[Loan Amount]]&lt;12000), "Approved", "Denied"))</f>
+        <v>Denied</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="67" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="67">
+        <v>750</v>
+      </c>
+      <c r="D5" s="69">
+        <v>25000</v>
+      </c>
+      <c r="E5" s="67" t="s">
+        <v>98</v>
+      </c>
+      <c r="F5" t="str">
+        <f>IF(Table5[[#This Row],[Credit Score]]&gt;700, "Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="G5" s="67" t="str">
+        <f>IF(OR(Table5[[#This Row],[Good Credit?]]="Yes", Table5[[#This Row],[Employement Status]]="Full-Time"), "Approved", IF(AND(C5&gt;650, Table5[[#This Row],[Loan Amount]]&lt;12000), "Approved", "Denied"))</f>
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="67" t="s">
+        <v>95</v>
+      </c>
+      <c r="C6" s="67">
+        <v>640</v>
+      </c>
+      <c r="D6" s="69">
+        <v>10000</v>
+      </c>
+      <c r="E6" s="67" t="s">
+        <v>100</v>
+      </c>
+      <c r="F6" t="str">
+        <f>IF(Table5[[#This Row],[Credit Score]]&gt;700, "Yes", "No")</f>
+        <v>No</v>
+      </c>
+      <c r="G6" s="67" t="str">
+        <f>IF(OR(Table5[[#This Row],[Good Credit?]]="Yes", Table5[[#This Row],[Employement Status]]="Full-Time"), "Approved", IF(AND(C6&gt;650, Table5[[#This Row],[Loan Amount]]&lt;12000), "Approved", "Denied"))</f>
+        <v>Denied</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="67" t="s">
+        <v>96</v>
+      </c>
+      <c r="C7" s="67">
+        <v>660</v>
+      </c>
+      <c r="D7" s="69">
+        <v>10000</v>
+      </c>
+      <c r="E7" s="67" t="s">
+        <v>99</v>
+      </c>
+      <c r="F7" t="str">
+        <f>IF(Table5[[#This Row],[Credit Score]]&gt;700, "Yes", "No")</f>
+        <v>No</v>
+      </c>
+      <c r="G7" s="67" t="str">
+        <f>IF(OR(Table5[[#This Row],[Good Credit?]]="Yes", Table5[[#This Row],[Employement Status]]="Full-Time"), "Approved", IF(AND(C7&gt;650, Table5[[#This Row],[Loan Amount]]&lt;12000), "Approved", "Denied"))</f>
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="67" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" s="67">
+        <v>710</v>
+      </c>
+      <c r="D8" s="69">
+        <v>18000</v>
+      </c>
+      <c r="E8" s="67" t="s">
+        <v>99</v>
+      </c>
+      <c r="F8" t="str">
+        <f>IF(Table5[[#This Row],[Credit Score]]&gt;700, "Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="G8" s="67" t="str">
+        <f>IF(OR(Table5[[#This Row],[Good Credit?]]="Yes", Table5[[#This Row],[Employement Status]]="Full-Time"), "Approved", IF(AND(C8&gt;650, Table5[[#This Row],[Loan Amount]]&lt;12000), "Approved", "Denied"))</f>
+        <v>Approved</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="C3:C8">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>$F3="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3:G8">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"Approved"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:G8">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"Denied"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{227D486A-352E-4CA0-80E8-EAB3033E6718}">
+  <dimension ref="B2:E12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="67" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" s="67" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="67" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" s="67" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="2">
+        <f ca="1">RANDBETWEEN(250, 3200)</f>
+        <v>1122</v>
+      </c>
+      <c r="E3" s="81">
+        <f ca="1">RANDBETWEEN(0, 2)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D4" s="2">
+        <f t="shared" ref="D4:D12" ca="1" si="0">RANDBETWEEN(250, 3200)</f>
+        <v>1228</v>
+      </c>
+      <c r="E4" s="81">
+        <f t="shared" ref="E3:E12" ca="1" si="1">RANDBETWEEN(0, 2)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D5" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>2326</v>
+      </c>
+      <c r="E5" s="81">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>825</v>
+      </c>
+      <c r="E6" s="81">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>1767</v>
+      </c>
+      <c r="E7" s="81">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" t="s">
+        <v>117</v>
+      </c>
+      <c r="D8" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>2430</v>
+      </c>
+      <c r="E8" s="81">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>2546</v>
+      </c>
+      <c r="E9" s="81">
+        <f t="shared" ca="1" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>109</v>
+      </c>
+      <c r="C10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>2063</v>
+      </c>
+      <c r="E10" s="81">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>2377</v>
+      </c>
+      <c r="E11" s="81">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>111</v>
+      </c>
+      <c r="C12" t="s">
+        <v>121</v>
+      </c>
+      <c r="D12" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>1273</v>
+      </c>
+      <c r="E12" s="81">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E0303D7-B63C-4C14-ADB0-194A7F9BABAD}">
   <dimension ref="B2:E6"/>
@@ -3008,240 +4848,240 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="75"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="56" t="s">
+      <c r="A2" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56" t="s">
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56" t="s">
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
+      <c r="J2" s="70"/>
+      <c r="K2" s="70"/>
+      <c r="L2" s="70"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="57">
+      <c r="A3" s="71">
         <v>46144</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="59">
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="73">
         <v>250.25</v>
       </c>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="58"/>
-      <c r="L3" s="58"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="72"/>
+      <c r="J3" s="72"/>
+      <c r="K3" s="72"/>
+      <c r="L3" s="72"/>
       <c r="N3" s="11" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="57">
+      <c r="A4" s="71">
         <v>46145</v>
       </c>
-      <c r="B4" s="58"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="59">
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="73">
         <v>300</v>
       </c>
-      <c r="F4" s="59"/>
-      <c r="G4" s="59"/>
-      <c r="H4" s="59"/>
-      <c r="I4" s="60">
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="74">
         <f>(E4-E3)/E3</f>
         <v>0.19880119880119881</v>
       </c>
-      <c r="J4" s="60"/>
-      <c r="K4" s="60"/>
-      <c r="L4" s="60"/>
+      <c r="J4" s="74"/>
+      <c r="K4" s="74"/>
+      <c r="L4" s="74"/>
       <c r="N4" s="10">
         <f>AVERAGE(I4:L11)</f>
         <v>-8.1596436336491718E-2</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="57">
+      <c r="A5" s="71">
         <v>46146</v>
       </c>
-      <c r="B5" s="58"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="59">
+      <c r="B5" s="72"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="73">
         <v>350.15</v>
       </c>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="60">
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="74">
         <f>(E5-E4)/E4</f>
         <v>0.1671666666666666</v>
       </c>
-      <c r="J5" s="60"/>
-      <c r="K5" s="60"/>
-      <c r="L5" s="60"/>
+      <c r="J5" s="74"/>
+      <c r="K5" s="74"/>
+      <c r="L5" s="74"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="57">
+      <c r="A6" s="71">
         <v>46147</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="59">
+      <c r="B6" s="72"/>
+      <c r="C6" s="72"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="73">
         <v>650.5</v>
       </c>
-      <c r="F6" s="59"/>
-      <c r="G6" s="59"/>
-      <c r="H6" s="59"/>
-      <c r="I6" s="60">
+      <c r="F6" s="73"/>
+      <c r="G6" s="73"/>
+      <c r="H6" s="73"/>
+      <c r="I6" s="74">
         <f>(E6-E5)/E5</f>
         <v>0.85777523918320731</v>
       </c>
-      <c r="J6" s="60"/>
-      <c r="K6" s="60"/>
-      <c r="L6" s="60"/>
+      <c r="J6" s="74"/>
+      <c r="K6" s="74"/>
+      <c r="L6" s="74"/>
       <c r="N6" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="57">
+      <c r="A7" s="71">
         <v>46148</v>
       </c>
-      <c r="B7" s="58"/>
-      <c r="C7" s="58"/>
-      <c r="D7" s="58"/>
-      <c r="E7" s="59">
+      <c r="B7" s="72"/>
+      <c r="C7" s="72"/>
+      <c r="D7" s="72"/>
+      <c r="E7" s="73">
         <v>600.35</v>
       </c>
-      <c r="F7" s="59"/>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
-      <c r="I7" s="60">
+      <c r="F7" s="73"/>
+      <c r="G7" s="73"/>
+      <c r="H7" s="73"/>
+      <c r="I7" s="74">
         <f t="shared" ref="I7:I10" si="0">(E7-E6)/E6</f>
         <v>-7.7094542659492657E-2</v>
       </c>
-      <c r="J7" s="60"/>
-      <c r="K7" s="60"/>
-      <c r="L7" s="60"/>
+      <c r="J7" s="74"/>
+      <c r="K7" s="74"/>
+      <c r="L7" s="74"/>
       <c r="N7" s="12" t="str">
         <f>IF(N4&gt;0,"Positive","Negative")</f>
         <v>Negative</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="57">
+      <c r="A8" s="71">
         <v>46149</v>
       </c>
-      <c r="B8" s="58"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="58"/>
-      <c r="E8" s="59">
+      <c r="B8" s="72"/>
+      <c r="C8" s="72"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="73">
         <v>150.19999999999999</v>
       </c>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="59"/>
-      <c r="I8" s="60">
+      <c r="F8" s="73"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="73"/>
+      <c r="I8" s="74">
         <f t="shared" si="0"/>
         <v>-0.74981260931123517</v>
       </c>
-      <c r="J8" s="60"/>
-      <c r="K8" s="60"/>
-      <c r="L8" s="60"/>
+      <c r="J8" s="74"/>
+      <c r="K8" s="74"/>
+      <c r="L8" s="74"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="57">
+      <c r="A9" s="71">
         <v>46150</v>
       </c>
-      <c r="B9" s="58"/>
-      <c r="C9" s="58"/>
-      <c r="D9" s="58"/>
-      <c r="E9" s="59">
+      <c r="B9" s="72"/>
+      <c r="C9" s="72"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="73">
         <v>55.5</v>
       </c>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
-      <c r="I9" s="60">
+      <c r="F9" s="73"/>
+      <c r="G9" s="73"/>
+      <c r="H9" s="73"/>
+      <c r="I9" s="74">
         <f t="shared" si="0"/>
         <v>-0.6304926764314247</v>
       </c>
-      <c r="J9" s="60"/>
-      <c r="K9" s="60"/>
-      <c r="L9" s="60"/>
+      <c r="J9" s="74"/>
+      <c r="K9" s="74"/>
+      <c r="L9" s="74"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="57">
+      <c r="A10" s="71">
         <v>46151</v>
       </c>
-      <c r="B10" s="58"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="58"/>
-      <c r="E10" s="59">
+      <c r="B10" s="72"/>
+      <c r="C10" s="72"/>
+      <c r="D10" s="72"/>
+      <c r="E10" s="73">
         <v>80.5</v>
       </c>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="59"/>
-      <c r="I10" s="60">
+      <c r="F10" s="73"/>
+      <c r="G10" s="73"/>
+      <c r="H10" s="73"/>
+      <c r="I10" s="74">
         <f t="shared" si="0"/>
         <v>0.45045045045045046</v>
       </c>
-      <c r="J10" s="60"/>
-      <c r="K10" s="60"/>
-      <c r="L10" s="60"/>
+      <c r="J10" s="74"/>
+      <c r="K10" s="74"/>
+      <c r="L10" s="74"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="57">
+      <c r="A11" s="71">
         <v>46152</v>
       </c>
-      <c r="B11" s="58"/>
-      <c r="C11" s="58"/>
-      <c r="D11" s="58"/>
-      <c r="E11" s="59">
+      <c r="B11" s="72"/>
+      <c r="C11" s="72"/>
+      <c r="D11" s="72"/>
+      <c r="E11" s="73">
         <v>10.5</v>
       </c>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="59"/>
-      <c r="I11" s="60">
+      <c r="F11" s="73"/>
+      <c r="G11" s="73"/>
+      <c r="H11" s="73"/>
+      <c r="I11" s="74">
         <f t="shared" ref="I11" si="1">(E11-E10)/E10</f>
         <v>-0.86956521739130432</v>
       </c>
-      <c r="J11" s="60"/>
-      <c r="K11" s="60"/>
-      <c r="L11" s="60"/>
+      <c r="J11" s="74"/>
+      <c r="K11" s="74"/>
+      <c r="L11" s="74"/>
     </row>
   </sheetData>
   <mergeCells count="31">
@@ -3556,27 +5396,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="76" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="63" t="s">
+      <c r="C1" s="77" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63" t="s">
+      <c r="D1" s="77"/>
+      <c r="E1" s="77" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="63"/>
-      <c r="G1" s="62" t="s">
+      <c r="F1" s="77"/>
+      <c r="G1" s="76" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="62"/>
-      <c r="B2" s="62"/>
+      <c r="A2" s="76"/>
+      <c r="B2" s="76"/>
       <c r="C2" s="21" t="s">
         <v>33</v>
       </c>
@@ -3589,7 +5429,7 @@
       <c r="F2" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="62"/>
+      <c r="G2" s="76"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
@@ -3597,11 +5437,11 @@
       </c>
       <c r="B3" s="24">
         <f ca="1">RANDBETWEEN(10, 50)</f>
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C3" s="30">
         <f ca="1">RANDBETWEEN(2, 10)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D3" s="22">
         <f ca="1">RANDBETWEEN(2, 10)</f>
@@ -3609,15 +5449,15 @@
       </c>
       <c r="E3" s="29">
         <f ca="1">$B3*C3</f>
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F3" s="35">
         <f ca="1">$B3*D3</f>
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="G3" s="38">
         <f ca="1">(E3+F3)/(E$8+F$8)</f>
-        <v>0.14996591683708249</v>
+        <v>9.6106456382454408E-2</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -3626,27 +5466,27 @@
       </c>
       <c r="B4" s="24">
         <f t="shared" ref="B4:B7" ca="1" si="0">RANDBETWEEN(10, 50)</f>
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C4" s="31">
         <f t="shared" ref="C4:D7" ca="1" si="1">RANDBETWEEN(2, 10)</f>
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D4" s="25">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E4" s="29">
         <f t="shared" ref="E4:F7" ca="1" si="2">$B4*C4</f>
-        <v>96</v>
+        <v>280</v>
       </c>
       <c r="F4" s="36">
         <f t="shared" ca="1" si="2"/>
-        <v>288</v>
+        <v>120</v>
       </c>
       <c r="G4" s="38">
         <f ca="1">(E4+F4)/(E$8+F$8)</f>
-        <v>0.26175869120654399</v>
+        <v>0.19714144898965008</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -3655,27 +5495,27 @@
       </c>
       <c r="B5" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="C5" s="31">
         <f t="shared" ca="1" si="1"/>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D5" s="28">
         <f t="shared" ca="1" si="1"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E5" s="29">
         <f t="shared" ca="1" si="2"/>
-        <v>130</v>
+        <v>245</v>
       </c>
       <c r="F5" s="35">
         <f t="shared" ca="1" si="2"/>
-        <v>117</v>
+        <v>490</v>
       </c>
       <c r="G5" s="38">
         <f t="shared" ref="G5:G7" ca="1" si="3">(E5+F5)/(E$8+F$8)</f>
-        <v>0.16837082481254259</v>
+        <v>0.36224741251848203</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -3684,27 +5524,27 @@
       </c>
       <c r="B6" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C6" s="26">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D6" s="25">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E6" s="29">
         <f t="shared" ca="1" si="2"/>
-        <v>64</v>
+        <v>333</v>
       </c>
       <c r="F6" s="35">
         <f t="shared" ca="1" si="2"/>
-        <v>192</v>
+        <v>111</v>
       </c>
       <c r="G6" s="38">
         <f t="shared" ca="1" si="3"/>
-        <v>0.17450579413769599</v>
+        <v>0.21882700837851157</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -3713,27 +5553,27 @@
       </c>
       <c r="B7" s="33">
         <f t="shared" ca="1" si="0"/>
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="C7" s="32">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D7" s="27">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E7" s="29">
         <f t="shared" ca="1" si="2"/>
-        <v>225</v>
+        <v>119</v>
       </c>
       <c r="F7" s="35">
         <f t="shared" ca="1" si="2"/>
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G7" s="38">
         <f t="shared" ca="1" si="3"/>
-        <v>0.24539877300613497</v>
+        <v>0.12567767373090191</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -3745,11 +5585,11 @@
       <c r="D8" s="34"/>
       <c r="E8" s="37">
         <f ca="1">SUM(E3:E7)</f>
-        <v>575</v>
+        <v>1052</v>
       </c>
       <c r="F8" s="37">
         <f ca="1">SUM(F3:F7)</f>
-        <v>892</v>
+        <v>977</v>
       </c>
       <c r="G8" s="34"/>
     </row>
@@ -3787,10 +5627,10 @@
       <c r="C1" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="64" t="s">
+      <c r="F1" s="78" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="64"/>
+      <c r="G1" s="78"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="51" t="s">
@@ -3801,14 +5641,14 @@
       </c>
       <c r="C2" s="41">
         <f ca="1">RANDBETWEEN(500, 1000)</f>
-        <v>892</v>
+        <v>565</v>
       </c>
       <c r="F2" s="45" t="s">
         <v>48</v>
       </c>
       <c r="G2" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F2, $C$2:$C$9)</f>
-        <v>1533</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -3820,14 +5660,14 @@
       </c>
       <c r="C3" s="44">
         <f t="shared" ref="C3:C9" ca="1" si="0">RANDBETWEEN(500, 1000)</f>
-        <v>690</v>
+        <v>961</v>
       </c>
       <c r="F3" s="34" t="s">
         <v>50</v>
       </c>
       <c r="G3" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F3)</f>
-        <v>598</v>
+        <v>513</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -3839,14 +5679,14 @@
       </c>
       <c r="C4" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>621</v>
+        <v>630</v>
       </c>
       <c r="F4" s="34" t="s">
         <v>51</v>
       </c>
       <c r="G4" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F4)</f>
-        <v>935</v>
+        <v>548</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -3858,14 +5698,14 @@
       </c>
       <c r="C5" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>641</v>
+        <v>694</v>
       </c>
       <c r="F5" s="45" t="s">
         <v>46</v>
       </c>
       <c r="G5" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F5, $C$2:$C$9)</f>
-        <v>1582</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -3877,14 +5717,14 @@
       </c>
       <c r="C6" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>598</v>
+        <v>513</v>
       </c>
       <c r="F6" s="34" t="s">
         <v>50</v>
       </c>
       <c r="G6" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F6)</f>
-        <v>892</v>
+        <v>565</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -3896,14 +5736,14 @@
       </c>
       <c r="C7" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>935</v>
+        <v>548</v>
       </c>
       <c r="F7" s="34" t="s">
         <v>51</v>
       </c>
       <c r="G7" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F7)</f>
-        <v>690</v>
+        <v>961</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -3915,14 +5755,14 @@
       </c>
       <c r="C8" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>898</v>
+        <v>926</v>
       </c>
       <c r="F8" s="45" t="s">
         <v>47</v>
       </c>
       <c r="G8" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F8, $C$2:$C$9)</f>
-        <v>1262</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -3934,14 +5774,14 @@
       </c>
       <c r="C9" s="42">
         <f t="shared" ca="1" si="0"/>
-        <v>811</v>
+        <v>613</v>
       </c>
       <c r="F9" s="34" t="s">
         <v>50</v>
       </c>
       <c r="G9" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F9)</f>
-        <v>621</v>
+        <v>630</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -3950,7 +5790,7 @@
       </c>
       <c r="G10" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F10)</f>
-        <v>641</v>
+        <v>694</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -3959,7 +5799,7 @@
       </c>
       <c r="G11" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F11, $C$2:$C$9)</f>
-        <v>1709</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -3968,7 +5808,7 @@
       </c>
       <c r="G12" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F12)</f>
-        <v>898</v>
+        <v>926</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -3977,7 +5817,7 @@
       </c>
       <c r="G13" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F13)</f>
-        <v>811</v>
+        <v>613</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -3986,7 +5826,7 @@
       </c>
       <c r="G14" s="43">
         <f ca="1">SUM(G2,G5,G8,G11)</f>
-        <v>6086</v>
+        <v>5450</v>
       </c>
     </row>
   </sheetData>
@@ -4010,172 +5850,172 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="66" t="s">
+      <c r="C1" s="57" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="66" t="s">
+      <c r="D1" s="57" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="67" t="s">
+      <c r="E1" s="58" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="68" t="s">
+      <c r="F1" s="59" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="2" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="60" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="69" t="s">
+      <c r="C2" s="60" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="69" t="s">
+      <c r="D2" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="E2" s="70">
+      <c r="E2" s="61">
         <v>60000</v>
       </c>
-      <c r="F2" s="71">
+      <c r="F2" s="62">
         <f>DATE(2026, 10, 5)</f>
         <v>46300</v>
       </c>
     </row>
     <row r="3" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="C3" s="69" t="s">
+      <c r="C3" s="60" t="s">
         <v>72</v>
       </c>
-      <c r="D3" s="69" t="s">
+      <c r="D3" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="70">
+      <c r="E3" s="61">
         <v>50000</v>
       </c>
-      <c r="F3" s="71">
+      <c r="F3" s="62">
         <f>DATE(2026, 4, 7)</f>
         <v>46119</v>
       </c>
     </row>
     <row r="4" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="60" t="s">
         <v>61</v>
       </c>
-      <c r="C4" s="69" t="s">
+      <c r="C4" s="60" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="69" t="s">
+      <c r="D4" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="E4" s="70">
+      <c r="E4" s="61">
         <v>25000</v>
       </c>
-      <c r="F4" s="71">
+      <c r="F4" s="62">
         <f>DATE(2026, 8, 7)</f>
         <v>46241</v>
       </c>
     </row>
     <row r="5" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="69" t="s">
+      <c r="B5" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="69" t="s">
+      <c r="C5" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="D5" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="E5" s="70">
+      <c r="E5" s="61">
         <v>15000</v>
       </c>
-      <c r="F5" s="71">
+      <c r="F5" s="62">
         <f>DATE(2026, 5, 8)</f>
         <v>46150</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="69" t="s">
+      <c r="B6" s="60" t="s">
         <v>62</v>
       </c>
-      <c r="C6" s="69" t="s">
+      <c r="C6" s="60" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="69" t="s">
+      <c r="D6" s="60" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="70">
+      <c r="E6" s="61">
         <v>10000</v>
       </c>
-      <c r="F6" s="71">
+      <c r="F6" s="62">
         <f>DATE(2026, 9, 7)</f>
         <v>46272</v>
       </c>
     </row>
     <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="69" t="s">
+      <c r="B7" s="60" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="69" t="s">
+      <c r="C7" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="D7" s="69" t="s">
+      <c r="D7" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="70">
+      <c r="E7" s="61">
         <v>7500</v>
       </c>
-      <c r="F7" s="71">
+      <c r="F7" s="62">
         <f>DATE(2026, 5, 7)</f>
         <v>46149</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="69" t="s">
+      <c r="B8" s="60" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="69" t="s">
+      <c r="C8" s="60" t="s">
         <v>66</v>
       </c>
-      <c r="D8" s="69" t="s">
+      <c r="D8" s="60" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="70">
+      <c r="E8" s="61">
         <v>7000</v>
       </c>
-      <c r="F8" s="71">
+      <c r="F8" s="62">
         <f>DATE(2026, 5, 7)</f>
         <v>46149</v>
       </c>
     </row>
     <row r="9" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="72" t="s">
+      <c r="B9" s="63" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="72" t="s">
+      <c r="C9" s="63" t="s">
         <v>67</v>
       </c>
-      <c r="D9" s="72" t="s">
+      <c r="D9" s="63" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="73">
+      <c r="E9" s="64">
         <v>6000</v>
       </c>
-      <c r="F9" s="74">
+      <c r="F9" s="65">
         <f>DATE(2026, 6, 6)</f>
         <v>46179</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C12" s="75" t="s">
+      <c r="C12" s="79" t="s">
         <v>74</v>
       </c>
-      <c r="D12" s="75"/>
-      <c r="E12" s="76">
+      <c r="D12" s="79"/>
+      <c r="E12" s="66">
         <f>SUM(JLoka_Investors[INVESTMENT AMOUNT (USD)])</f>
         <v>180500</v>
       </c>
@@ -4213,25 +6053,25 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B2" s="78" t="s">
+      <c r="B2" s="80" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="77"/>
-    </row>
-    <row r="3" spans="2:6" s="77" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="77" t="s">
+      <c r="C2" s="80"/>
+      <c r="D2" s="80"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="67"/>
+    </row>
+    <row r="3" spans="2:6" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="67" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="77" t="s">
+      <c r="C3" s="67" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="77" t="s">
+      <c r="D3" s="67" t="s">
         <v>78</v>
       </c>
-      <c r="E3" s="77" t="s">
+      <c r="E3" s="67" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4241,15 +6081,15 @@
       </c>
       <c r="C4" s="3">
         <f ca="1">RAND()</f>
-        <v>0.74632334827253011</v>
+        <v>0.82725387354161772</v>
       </c>
       <c r="D4" s="3">
         <f t="shared" ref="D4:E4" ca="1" si="0">RAND()</f>
-        <v>7.6764236190715374E-2</v>
+        <v>0.80017116372062791</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.59766622878496245</v>
+        <v>0.20801938180659352</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -4258,15 +6098,15 @@
       </c>
       <c r="C5" s="3">
         <f t="shared" ref="C5:E14" ca="1" si="1">RAND()</f>
-        <v>0.96726538064451084</v>
+        <v>0.98231634059209239</v>
       </c>
       <c r="D5" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>5.4354528886120357E-2</v>
+        <v>0.59857569406591837</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.35034220588725351</v>
+        <v>5.8172409636129241E-2</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
@@ -4275,15 +6115,15 @@
       </c>
       <c r="C6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.34234357821502415</v>
+        <v>0.92177328897518906</v>
       </c>
       <c r="D6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.28344606593773036</v>
+        <v>0.62960068734179109</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.69553741865844598</v>
+        <v>0.47613209032723569</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
@@ -4292,15 +6132,15 @@
       </c>
       <c r="C7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.6802225754616299</v>
+        <v>6.8127943760001086E-2</v>
       </c>
       <c r="D7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.71322647348581636</v>
+        <v>0.91148131598852689</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.58331324969536502</v>
+        <v>0.33943465465660472</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
@@ -4309,15 +6149,15 @@
       </c>
       <c r="C8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.41154429073134569</v>
+        <v>0.36546159306277792</v>
       </c>
       <c r="D8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.24424704666357588</v>
+        <v>0.49768864602230933</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>4.5648847882053256E-2</v>
+        <v>0.56689538950625051</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
@@ -4326,15 +6166,15 @@
       </c>
       <c r="C9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>2.8166285419759518E-3</v>
+        <v>7.0132702277079795E-2</v>
       </c>
       <c r="D9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>9.6777844968651827E-2</v>
+        <v>0.39161580424131404</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.70430520884159553</v>
+        <v>0.70946690247282718</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
@@ -4343,15 +6183,15 @@
       </c>
       <c r="C10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.55602648328598325</v>
+        <v>0.29363415525332215</v>
       </c>
       <c r="D10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.52020423431596585</v>
+        <v>3.4430219338273838E-2</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.34173611134409643</v>
+        <v>0.48517707387830089</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
@@ -4360,15 +6200,15 @@
       </c>
       <c r="C11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.72204098578482745</v>
+        <v>0.57614710490615306</v>
       </c>
       <c r="D11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.32085133206821126</v>
+        <v>0.88951744204066985</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.38026533146699537</v>
+        <v>0.34191490610491293</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
@@ -4377,15 +6217,15 @@
       </c>
       <c r="C12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.75989775807371251</v>
+        <v>0.42653486070031332</v>
       </c>
       <c r="D12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.47604524511131241</v>
+        <v>0.21054797943785342</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.61216195487650615</v>
+        <v>0.75340815882757395</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
@@ -4394,15 +6234,15 @@
       </c>
       <c r="C13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.36214243666635559</v>
+        <v>0.27532486384594812</v>
       </c>
       <c r="D13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.96824967018629216</v>
+        <v>0.29914873161213729</v>
       </c>
       <c r="E13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.94629380652869344</v>
+        <v>0.73473476496323886</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
@@ -4411,15 +6251,15 @@
       </c>
       <c r="C14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>8.0557715692428644E-3</v>
+        <v>0.39228657162766789</v>
       </c>
       <c r="D14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.99040654877882894</v>
+        <v>0.72402950173284431</v>
       </c>
       <c r="E14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.8497834350972423</v>
+        <v>6.5175240099631937E-3</v>
       </c>
     </row>
   </sheetData>
@@ -4432,4 +6272,62 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8721280-4213-4B53-9A0B-5F17D269CBD8}">
+  <dimension ref="B2:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="68">
+        <v>0.60699999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="68">
+        <v>0.29299999999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="68">
+        <v>6.5000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="68">
+        <v>3.5000000000000003E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adding Finance examples with Excel and XLOOKUP & VLOOKUP
</commit_message>
<xml_diff>
--- a/Excel-Finance/JLoka-Finance-01.xlsx
+++ b/Excel-Finance/JLoka-Finance-01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\books-and-tutorials\Finance-Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\j-l-data-science-data-analytics\Excel-Finance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F6522C-427F-48A1-9567-6B6BBB9E8212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602BA44E-F45F-417D-8C06-199DBCCCD0FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="4" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="Sheet9" sheetId="9" r:id="rId9"/>
     <sheet name="Sheet10" sheetId="10" r:id="rId10"/>
     <sheet name="Sheet11" sheetId="11" r:id="rId11"/>
+    <sheet name="With XLOOKUP" sheetId="12" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet7!$B$1:$F$9</definedName>
@@ -37,8 +38,8 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicerCache r:id="rId12"/>
         <x14:slicerCache r:id="rId13"/>
+        <x14:slicerCache r:id="rId14"/>
       </x15:slicerCaches>
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="116">
   <si>
     <t>Sunday</t>
   </si>
@@ -376,24 +377,6 @@
   </si>
   <si>
     <t>Jloka-04</t>
-  </si>
-  <si>
-    <t>Jloka-05</t>
-  </si>
-  <si>
-    <t>Jloka-06</t>
-  </si>
-  <si>
-    <t>Jloka-07</t>
-  </si>
-  <si>
-    <t>Jloka-08</t>
-  </si>
-  <si>
-    <t>Jloka-09</t>
-  </si>
-  <si>
-    <t>Jloka-10</t>
   </si>
   <si>
     <t>Jloka-100</t>
@@ -1004,6 +987,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1037,16 +1023,13 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="35">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1065,6 +1048,124 @@
           <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1286,11 +1387,42 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1312,14 +1444,25 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1550,31 +1693,31 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.92177328897518906</c:v>
+                  <c:v>0.17562438708328187</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.8127943760001086E-2</c:v>
+                  <c:v>0.97179011742401034</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.36546159306277792</c:v>
+                  <c:v>0.84749572115146177</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.0132702277079795E-2</c:v>
+                  <c:v>0.93566798383572247</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.29363415525332215</c:v>
+                  <c:v>0.1433999468745274</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.57614710490615306</c:v>
+                  <c:v>0.21221459352036331</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.42653486070031332</c:v>
+                  <c:v>4.7972957196397492E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.27532486384594812</c:v>
+                  <c:v>0.72753524488705212</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.39228657162766789</c:v>
+                  <c:v>0.89667820846322988</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1714,31 +1857,31 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.62960068734179109</c:v>
+                  <c:v>0.9163764591219179</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.91148131598852689</c:v>
+                  <c:v>0.86700995900552902</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.49768864602230933</c:v>
+                  <c:v>0.14018279942935719</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.39161580424131404</c:v>
+                  <c:v>0.92855436625288845</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.4430219338273838E-2</c:v>
+                  <c:v>0.63410830731845791</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.88951744204066985</c:v>
+                  <c:v>0.30477536836824548</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.21054797943785342</c:v>
+                  <c:v>0.63336008174203462</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.29914873161213729</c:v>
+                  <c:v>0.44769928553516947</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.72402950173284431</c:v>
+                  <c:v>0.3584885461089784</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1878,31 +2021,31 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.47613209032723569</c:v>
+                  <c:v>0.98052310491075534</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.33943465465660472</c:v>
+                  <c:v>0.53703235256206727</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.56689538950625051</c:v>
+                  <c:v>0.16890054256540799</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.70946690247282718</c:v>
+                  <c:v>0.1460052583933078</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.48517707387830089</c:v>
+                  <c:v>0.6021723468059248</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.34191490610491293</c:v>
+                  <c:v>5.9313688358269889E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.75340815882757395</c:v>
+                  <c:v>0.19399467707450213</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.73473476496323886</c:v>
+                  <c:v>0.22340416548027076</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6.5175240099631937E-3</c:v>
+                  <c:v>6.1928356350029135E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3952,7 +4095,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{385DC015-9960-47FA-A637-6B66C3CB4FFA}" name="JLoka_Investors" displayName="JLoka_Investors" ref="B1:F9" totalsRowShown="0" dataDxfId="15" tableBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{385DC015-9960-47FA-A637-6B66C3CB4FFA}" name="JLoka_Investors" displayName="JLoka_Investors" ref="B1:F9" totalsRowShown="0" dataDxfId="28" tableBorderDxfId="27">
   <autoFilter ref="B1:F9" xr:uid="{22AB70FF-96FA-4025-A517-8BDE3ECE5EBF}">
     <filterColumn colId="2">
       <filters>
@@ -3961,28 +4104,28 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{0BE1A407-37E2-45E1-A4B9-6EE27C852CA8}" name="INVESTOR_ID" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{F40E02B0-B4B8-4130-A683-00045FEF2BC6}" name="INVESTOR_NAME" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{EB541472-54EA-4246-959A-8F16F8FDA58F}" name="COMPANY_NAME" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{B149ED9E-81EF-4313-90DA-EDCF3ACBE03C}" name="INVESTMENT AMOUNT (USD)" dataDxfId="10" dataCellStyle="Currency"/>
-    <tableColumn id="5" xr3:uid="{5C700949-A13F-423E-81D1-C89753142DF7}" name="INVESTMENT_DATE" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{0BE1A407-37E2-45E1-A4B9-6EE27C852CA8}" name="INVESTOR_ID" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{F40E02B0-B4B8-4130-A683-00045FEF2BC6}" name="INVESTOR_NAME" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{EB541472-54EA-4246-959A-8F16F8FDA58F}" name="COMPANY_NAME" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{B149ED9E-81EF-4313-90DA-EDCF3ACBE03C}" name="INVESTMENT AMOUNT (USD)" dataDxfId="23" dataCellStyle="Currency"/>
+    <tableColumn id="5" xr3:uid="{5C700949-A13F-423E-81D1-C89753142DF7}" name="INVESTMENT_DATE" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E0111534-CC78-4AAC-9FB0-08AB9DCECE24}" name="Table4" displayName="Table4" ref="B3:E14" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7" dataCellStyle="Percent">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E0111534-CC78-4AAC-9FB0-08AB9DCECE24}" name="Table4" displayName="Table4" ref="B3:E14" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" dataCellStyle="Percent">
   <autoFilter ref="B3:E14" xr:uid="{E0111534-CC78-4AAC-9FB0-08AB9DCECE24}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{B5AEA49B-906B-4BA3-9E02-DF265E516312}" name="Year"/>
-    <tableColumn id="2" xr3:uid="{8C94788E-9FB3-46B0-A805-B97EFDDC36C5}" name="Jloka-01" dataDxfId="6" dataCellStyle="Percent">
+    <tableColumn id="2" xr3:uid="{8C94788E-9FB3-46B0-A805-B97EFDDC36C5}" name="Jloka-01" dataDxfId="19" dataCellStyle="Percent">
       <calculatedColumnFormula>RAND()</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A2693482-C7C8-4B05-9865-B12ABE5CC110}" name="Jloka-02" dataDxfId="5" dataCellStyle="Percent">
+    <tableColumn id="3" xr3:uid="{A2693482-C7C8-4B05-9865-B12ABE5CC110}" name="Jloka-02" dataDxfId="18" dataCellStyle="Percent">
       <calculatedColumnFormula>RAND()</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8F26A52C-2531-497C-A839-2A770D581E4E}" name="Jloka-03" dataDxfId="4" dataCellStyle="Percent">
+    <tableColumn id="4" xr3:uid="{8F26A52C-2531-497C-A839-2A770D581E4E}" name="Jloka-03" dataDxfId="17" dataCellStyle="Percent">
       <calculatedColumnFormula>RAND()</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3995,28 +4138,94 @@
   <autoFilter ref="B2:C6" xr:uid="{80A2B397-4223-4F15-9DB4-892BEE67AC07}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{C09EC9D1-D203-4F94-BBB0-27B52BD67348}" name="Investment Type"/>
-    <tableColumn id="2" xr3:uid="{DDA73600-5426-4CA3-8EA1-3D48A09909F0}" name="Portfolio Allocation" dataDxfId="3" dataCellStyle="Percent"/>
+    <tableColumn id="2" xr3:uid="{DDA73600-5426-4CA3-8EA1-3D48A09909F0}" name="Portfolio Allocation" dataDxfId="16" dataCellStyle="Percent"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{26F768BE-F4AC-48CD-9271-53238CC90A9E}" name="Table5" displayName="Table5" ref="B2:G8" totalsRowShown="0" headerRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{26F768BE-F4AC-48CD-9271-53238CC90A9E}" name="Table5" displayName="Table5" ref="B2:G8" totalsRowShown="0" headerRowDxfId="15">
   <autoFilter ref="B2:G8" xr:uid="{26F768BE-F4AC-48CD-9271-53238CC90A9E}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{CD0DE5D2-C8ED-45CF-8F5D-E6E88682B06A}" name="Applicant" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{89F30673-4126-482B-AFC9-E6FAD8DBE3F4}" name="Credit Score" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{4BC38630-914F-4BE8-9B0A-961F3FF855C4}" name="Loan Amount" dataDxfId="19" dataCellStyle="Currency"/>
-    <tableColumn id="4" xr3:uid="{7CE22975-ED55-49DD-B302-D5C876BF8196}" name="Employement Status" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{BD342C3D-5A81-4372-A781-AB1A62E26D7B}" name="Good Credit?" dataDxfId="17">
+    <tableColumn id="1" xr3:uid="{CD0DE5D2-C8ED-45CF-8F5D-E6E88682B06A}" name="Applicant" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{89F30673-4126-482B-AFC9-E6FAD8DBE3F4}" name="Credit Score" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{4BC38630-914F-4BE8-9B0A-961F3FF855C4}" name="Loan Amount" dataDxfId="12" dataCellStyle="Currency"/>
+    <tableColumn id="4" xr3:uid="{7CE22975-ED55-49DD-B302-D5C876BF8196}" name="Employement Status" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{BD342C3D-5A81-4372-A781-AB1A62E26D7B}" name="Good Credit?" dataDxfId="10">
       <calculatedColumnFormula>IF(Table5[[#This Row],[Credit Score]]&gt;700, "Yes", "No")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{14D8C1DF-DE7F-494A-8E09-15D4A0C38048}" name="Approved or Denied?" dataDxfId="16">
+    <tableColumn id="6" xr3:uid="{14D8C1DF-DE7F-494A-8E09-15D4A0C38048}" name="Approved or Denied?" dataDxfId="9">
       <calculatedColumnFormula>IF(OR(Table5[[#This Row],[Good Credit?]]="Yes", Table5[[#This Row],[Employement Status]]="Full-Time"), "Approved", IF(AND(C3&gt;650, Table5[[#This Row],[Loan Amount]]&lt;12000), "Approved", "Denied"))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D6776827-273F-4CF2-BBDD-3C1A235A406D}" name="Table1" displayName="Table1" ref="B2:E12" totalsRowShown="0" headerRowDxfId="8">
+  <autoFilter ref="B2:E12" xr:uid="{D6776827-273F-4CF2-BBDD-3C1A235A406D}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{6A18450A-3CA5-4EB5-8DD9-4859B5561889}" name="Ticker"/>
+    <tableColumn id="2" xr3:uid="{FA7BE9A2-00B3-4719-BE3C-20A682E122D9}" name="Company"/>
+    <tableColumn id="3" xr3:uid="{93EFFFCB-2911-497B-87A0-3A4DF10829DB}" name="Price" dataDxfId="7" dataCellStyle="Currency">
+      <calculatedColumnFormula>RANDBETWEEN(250, 3200)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{1545D519-F59F-4471-957F-E0327328561F}" name="Dividend" dataDxfId="6" dataCellStyle="Currency">
+      <calculatedColumnFormula>RANDBETWEEN(0, 2)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{523D5987-9D63-4495-A3E0-40C18910C1BB}" name="Table6" displayName="Table6" ref="G2:I6" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="G2:I6" xr:uid="{523D5987-9D63-4495-A3E0-40C18910C1BB}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{5F0DF985-326B-4188-9761-4EF834FAAC8F}" name="Ticker"/>
+    <tableColumn id="2" xr3:uid="{34F55C9B-69AE-404C-BCD4-52F70E9A9001}" name="Price" dataDxfId="4" dataCellStyle="Currency">
+      <calculatedColumnFormula>VLOOKUP($G3, Table1[], 3, FALSE)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{CB5E81CC-AE6E-4E52-BCE7-89190BAE3FC0}" name="Dividend" dataDxfId="3" dataCellStyle="Currency">
+      <calculatedColumnFormula>VLOOKUP($G3, Table1[], 4, FALSE)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{82E15C98-66B8-471C-A245-225B29CE147F}" name="Table18" displayName="Table18" ref="B2:E12" totalsRowShown="0" headerRowDxfId="34">
+  <autoFilter ref="B2:E12" xr:uid="{D6776827-273F-4CF2-BBDD-3C1A235A406D}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{6153BC4B-CB64-4AF3-8BDB-3C67B9222CA2}" name="Ticker"/>
+    <tableColumn id="2" xr3:uid="{52D14EC0-E80A-4AD1-B945-4AF713433E12}" name="Company"/>
+    <tableColumn id="3" xr3:uid="{1B82F8EC-F7E7-47A6-9E49-3400ACAAE6B6}" name="Price" dataDxfId="33" dataCellStyle="Currency">
+      <calculatedColumnFormula>RANDBETWEEN(250, 3200)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{EEAF0D74-71EA-45D2-A67A-FB1DFB7D91AE}" name="Dividend" dataDxfId="32" dataCellStyle="Currency">
+      <calculatedColumnFormula>RANDBETWEEN(0, 2)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{F24AB42E-2508-4FC6-9636-69F943E6AC52}" name="Table69" displayName="Table69" ref="G2:I6" totalsRowShown="0" headerRowDxfId="31">
+  <autoFilter ref="G2:I6" xr:uid="{523D5987-9D63-4495-A3E0-40C18910C1BB}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{51F24543-C1E6-46E0-9D99-BA4472C976F6}" name="Ticker"/>
+    <tableColumn id="2" xr3:uid="{D2E2C469-1439-4BE7-9808-48F853A4077B}" name="Price" dataDxfId="30" dataCellStyle="Currency">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Price], "Missing")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{E0FC8430-98AC-4152-B1BA-30813CCFBC65}" name="Dividend" dataDxfId="29" dataCellStyle="Currency">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Dividend], "Missing")</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -4563,16 +4772,19 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{227D486A-352E-4CA0-80E8-EAB3033E6718}">
-  <dimension ref="B2:E12"/>
+  <dimension ref="B2:I12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="13.7109375" customWidth="1"/>
     <col min="4" max="4" width="13.140625" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="7" max="7" width="19.85546875" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="67" t="s">
         <v>101</v>
       </c>
@@ -4585,163 +4797,216 @@
       <c r="E2" s="67" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G2" s="67" t="s">
+        <v>101</v>
+      </c>
+      <c r="H2" s="67" t="s">
+        <v>103</v>
+      </c>
+      <c r="I2" s="67" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>77</v>
       </c>
       <c r="C3" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D3" s="2">
         <f ca="1">RANDBETWEEN(250, 3200)</f>
-        <v>1122</v>
-      </c>
-      <c r="E3" s="81">
+        <v>1889</v>
+      </c>
+      <c r="E3" s="70">
         <f ca="1">RANDBETWEEN(0, 2)</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H3" s="2">
+        <f ca="1">VLOOKUP($G3, Table1[], 3, FALSE)</f>
+        <v>1889</v>
+      </c>
+      <c r="I3" s="2">
+        <f ca="1">VLOOKUP($G3, Table1[], 4, FALSE)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" ref="D4:D12" ca="1" si="0">RANDBETWEEN(250, 3200)</f>
-        <v>1228</v>
-      </c>
-      <c r="E4" s="81">
-        <f t="shared" ref="E3:E12" ca="1" si="1">RANDBETWEEN(0, 2)</f>
+        <v>2579</v>
+      </c>
+      <c r="E4" s="70">
+        <f t="shared" ref="E4:E12" ca="1" si="1">RANDBETWEEN(0, 2)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>78</v>
+      </c>
+      <c r="H4" s="2">
+        <f ca="1">VLOOKUP($G4, Table1[], 3, FALSE)</f>
+        <v>2579</v>
+      </c>
+      <c r="I4" s="2">
+        <f ca="1">VLOOKUP($G4, Table1[], 4, FALSE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D5" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>2326</v>
-      </c>
-      <c r="E5" s="81">
+        <v>2328</v>
+      </c>
+      <c r="E5" s="70">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="G5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H5" s="2">
+        <f ca="1">VLOOKUP($G5, Table1[], 3, FALSE)</f>
+        <v>3058</v>
+      </c>
+      <c r="I5" s="2">
+        <f ca="1">VLOOKUP($G5, Table1[], 4, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>1742</v>
+      </c>
+      <c r="E6" s="70">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="G6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H6" s="2">
+        <f ca="1">VLOOKUP($G6, Table1[], 3, FALSE)</f>
+        <v>1368</v>
+      </c>
+      <c r="I6" s="2">
+        <f ca="1">VLOOKUP($G6, Table1[], 4, FALSE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>2717</v>
+      </c>
+      <c r="E7" s="70">
         <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C6" t="s">
-        <v>115</v>
-      </c>
-      <c r="D6" s="2">
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D8" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>825</v>
-      </c>
-      <c r="E6" s="81">
+        <v>3058</v>
+      </c>
+      <c r="E8" s="70">
         <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C7" t="s">
-        <v>116</v>
-      </c>
-      <c r="D7" s="2">
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>1767</v>
-      </c>
-      <c r="E7" s="81">
+        <v>2576</v>
+      </c>
+      <c r="E9" s="70">
         <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" t="s">
-        <v>117</v>
-      </c>
-      <c r="D8" s="2">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D10" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>2430</v>
-      </c>
-      <c r="E8" s="81">
+        <v>2568</v>
+      </c>
+      <c r="E10" s="70">
         <f t="shared" ca="1" si="1"/>
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>108</v>
-      </c>
-      <c r="C9" t="s">
-        <v>118</v>
-      </c>
-      <c r="D9" s="2">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>2546</v>
-      </c>
-      <c r="E9" s="81">
+        <v>1368</v>
+      </c>
+      <c r="E11" s="70">
         <f t="shared" ca="1" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C10" t="s">
-        <v>119</v>
-      </c>
-      <c r="D10" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>2063</v>
-      </c>
-      <c r="E10" s="81">
-        <f t="shared" ca="1" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>110</v>
-      </c>
-      <c r="C11" t="s">
-        <v>120</v>
-      </c>
-      <c r="D11" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>2377</v>
-      </c>
-      <c r="E11" s="81">
-        <f t="shared" ca="1" si="1"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="C12" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D12" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>1273</v>
-      </c>
-      <c r="E12" s="81">
+        <v>2086</v>
+      </c>
+      <c r="E12" s="70">
         <f t="shared" ca="1" si="1"/>
         <v>2</v>
       </c>
@@ -4749,6 +5014,260 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12846ECA-6E1C-4031-BB27-C674131C97A8}">
+  <dimension ref="B2:I12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="7" max="7" width="19.85546875" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="67" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" s="67" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="67" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" s="67" t="s">
+        <v>104</v>
+      </c>
+      <c r="G2" s="67" t="s">
+        <v>101</v>
+      </c>
+      <c r="H2" s="67" t="s">
+        <v>103</v>
+      </c>
+      <c r="I2" s="67" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D3" s="2">
+        <f ca="1">RANDBETWEEN(250, 3200)</f>
+        <v>607</v>
+      </c>
+      <c r="E3" s="70">
+        <f ca="1">RANDBETWEEN(0, 2)</f>
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H3" s="2">
+        <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Price], "Missing")</f>
+        <v>607</v>
+      </c>
+      <c r="I3" s="2">
+        <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Dividend], "Missing")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="2">
+        <f t="shared" ref="D4:D12" ca="1" si="0">RANDBETWEEN(250, 3200)</f>
+        <v>2613</v>
+      </c>
+      <c r="E4" s="70">
+        <f t="shared" ref="E4:E12" ca="1" si="1">RANDBETWEEN(0, 2)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>78</v>
+      </c>
+      <c r="H4" s="2">
+        <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Price], "Missing")</f>
+        <v>2613</v>
+      </c>
+      <c r="I4" s="2">
+        <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Dividend], "Missing")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D5" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>769</v>
+      </c>
+      <c r="E5" s="70">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="G5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H5" s="2">
+        <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Price], "Missing")</f>
+        <v>732</v>
+      </c>
+      <c r="I5" s="2">
+        <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Dividend], "Missing")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>816</v>
+      </c>
+      <c r="E6" s="70">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H6" s="2">
+        <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Price], "Missing")</f>
+        <v>3071</v>
+      </c>
+      <c r="I6" s="2">
+        <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Dividend], "Missing")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>1890</v>
+      </c>
+      <c r="E7" s="70">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D8" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>732</v>
+      </c>
+      <c r="E8" s="70">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>3200</v>
+      </c>
+      <c r="E9" s="70">
+        <f t="shared" ca="1" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D10" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>2186</v>
+      </c>
+      <c r="E10" s="70">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>3071</v>
+      </c>
+      <c r="E11" s="70">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>1931</v>
+      </c>
+      <c r="E12" s="70">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -4848,240 +5367,240 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="76" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
-      <c r="H1" s="75"/>
-      <c r="I1" s="75"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="76"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70" t="s">
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70" t="s">
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="71">
+      <c r="A3" s="72">
         <v>46144</v>
       </c>
-      <c r="B3" s="72"/>
-      <c r="C3" s="72"/>
-      <c r="D3" s="72"/>
-      <c r="E3" s="73">
+      <c r="B3" s="73"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="74">
         <v>250.25</v>
       </c>
-      <c r="F3" s="73"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="73"/>
-      <c r="I3" s="72"/>
-      <c r="J3" s="72"/>
-      <c r="K3" s="72"/>
-      <c r="L3" s="72"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
+      <c r="I3" s="73"/>
+      <c r="J3" s="73"/>
+      <c r="K3" s="73"/>
+      <c r="L3" s="73"/>
       <c r="N3" s="11" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="71">
+      <c r="A4" s="72">
         <v>46145</v>
       </c>
-      <c r="B4" s="72"/>
-      <c r="C4" s="72"/>
-      <c r="D4" s="72"/>
-      <c r="E4" s="73">
+      <c r="B4" s="73"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="74">
         <v>300</v>
       </c>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="74">
+      <c r="F4" s="74"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
+      <c r="I4" s="75">
         <f>(E4-E3)/E3</f>
         <v>0.19880119880119881</v>
       </c>
-      <c r="J4" s="74"/>
-      <c r="K4" s="74"/>
-      <c r="L4" s="74"/>
+      <c r="J4" s="75"/>
+      <c r="K4" s="75"/>
+      <c r="L4" s="75"/>
       <c r="N4" s="10">
         <f>AVERAGE(I4:L11)</f>
         <v>-8.1596436336491718E-2</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="71">
+      <c r="A5" s="72">
         <v>46146</v>
       </c>
-      <c r="B5" s="72"/>
-      <c r="C5" s="72"/>
-      <c r="D5" s="72"/>
-      <c r="E5" s="73">
+      <c r="B5" s="73"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="74">
         <v>350.15</v>
       </c>
-      <c r="F5" s="73"/>
-      <c r="G5" s="73"/>
-      <c r="H5" s="73"/>
-      <c r="I5" s="74">
+      <c r="F5" s="74"/>
+      <c r="G5" s="74"/>
+      <c r="H5" s="74"/>
+      <c r="I5" s="75">
         <f>(E5-E4)/E4</f>
         <v>0.1671666666666666</v>
       </c>
-      <c r="J5" s="74"/>
-      <c r="K5" s="74"/>
-      <c r="L5" s="74"/>
+      <c r="J5" s="75"/>
+      <c r="K5" s="75"/>
+      <c r="L5" s="75"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="71">
+      <c r="A6" s="72">
         <v>46147</v>
       </c>
-      <c r="B6" s="72"/>
-      <c r="C6" s="72"/>
-      <c r="D6" s="72"/>
-      <c r="E6" s="73">
+      <c r="B6" s="73"/>
+      <c r="C6" s="73"/>
+      <c r="D6" s="73"/>
+      <c r="E6" s="74">
         <v>650.5</v>
       </c>
-      <c r="F6" s="73"/>
-      <c r="G6" s="73"/>
-      <c r="H6" s="73"/>
-      <c r="I6" s="74">
+      <c r="F6" s="74"/>
+      <c r="G6" s="74"/>
+      <c r="H6" s="74"/>
+      <c r="I6" s="75">
         <f>(E6-E5)/E5</f>
         <v>0.85777523918320731</v>
       </c>
-      <c r="J6" s="74"/>
-      <c r="K6" s="74"/>
-      <c r="L6" s="74"/>
+      <c r="J6" s="75"/>
+      <c r="K6" s="75"/>
+      <c r="L6" s="75"/>
       <c r="N6" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="71">
+      <c r="A7" s="72">
         <v>46148</v>
       </c>
-      <c r="B7" s="72"/>
-      <c r="C7" s="72"/>
-      <c r="D7" s="72"/>
-      <c r="E7" s="73">
+      <c r="B7" s="73"/>
+      <c r="C7" s="73"/>
+      <c r="D7" s="73"/>
+      <c r="E7" s="74">
         <v>600.35</v>
       </c>
-      <c r="F7" s="73"/>
-      <c r="G7" s="73"/>
-      <c r="H7" s="73"/>
-      <c r="I7" s="74">
+      <c r="F7" s="74"/>
+      <c r="G7" s="74"/>
+      <c r="H7" s="74"/>
+      <c r="I7" s="75">
         <f t="shared" ref="I7:I10" si="0">(E7-E6)/E6</f>
         <v>-7.7094542659492657E-2</v>
       </c>
-      <c r="J7" s="74"/>
-      <c r="K7" s="74"/>
-      <c r="L7" s="74"/>
+      <c r="J7" s="75"/>
+      <c r="K7" s="75"/>
+      <c r="L7" s="75"/>
       <c r="N7" s="12" t="str">
         <f>IF(N4&gt;0,"Positive","Negative")</f>
         <v>Negative</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="71">
+      <c r="A8" s="72">
         <v>46149</v>
       </c>
-      <c r="B8" s="72"/>
-      <c r="C8" s="72"/>
-      <c r="D8" s="72"/>
-      <c r="E8" s="73">
+      <c r="B8" s="73"/>
+      <c r="C8" s="73"/>
+      <c r="D8" s="73"/>
+      <c r="E8" s="74">
         <v>150.19999999999999</v>
       </c>
-      <c r="F8" s="73"/>
-      <c r="G8" s="73"/>
-      <c r="H8" s="73"/>
-      <c r="I8" s="74">
+      <c r="F8" s="74"/>
+      <c r="G8" s="74"/>
+      <c r="H8" s="74"/>
+      <c r="I8" s="75">
         <f t="shared" si="0"/>
         <v>-0.74981260931123517</v>
       </c>
-      <c r="J8" s="74"/>
-      <c r="K8" s="74"/>
-      <c r="L8" s="74"/>
+      <c r="J8" s="75"/>
+      <c r="K8" s="75"/>
+      <c r="L8" s="75"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="71">
+      <c r="A9" s="72">
         <v>46150</v>
       </c>
-      <c r="B9" s="72"/>
-      <c r="C9" s="72"/>
-      <c r="D9" s="72"/>
-      <c r="E9" s="73">
+      <c r="B9" s="73"/>
+      <c r="C9" s="73"/>
+      <c r="D9" s="73"/>
+      <c r="E9" s="74">
         <v>55.5</v>
       </c>
-      <c r="F9" s="73"/>
-      <c r="G9" s="73"/>
-      <c r="H9" s="73"/>
-      <c r="I9" s="74">
+      <c r="F9" s="74"/>
+      <c r="G9" s="74"/>
+      <c r="H9" s="74"/>
+      <c r="I9" s="75">
         <f t="shared" si="0"/>
         <v>-0.6304926764314247</v>
       </c>
-      <c r="J9" s="74"/>
-      <c r="K9" s="74"/>
-      <c r="L9" s="74"/>
+      <c r="J9" s="75"/>
+      <c r="K9" s="75"/>
+      <c r="L9" s="75"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="71">
+      <c r="A10" s="72">
         <v>46151</v>
       </c>
-      <c r="B10" s="72"/>
-      <c r="C10" s="72"/>
-      <c r="D10" s="72"/>
-      <c r="E10" s="73">
+      <c r="B10" s="73"/>
+      <c r="C10" s="73"/>
+      <c r="D10" s="73"/>
+      <c r="E10" s="74">
         <v>80.5</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="73"/>
-      <c r="H10" s="73"/>
-      <c r="I10" s="74">
+      <c r="F10" s="74"/>
+      <c r="G10" s="74"/>
+      <c r="H10" s="74"/>
+      <c r="I10" s="75">
         <f t="shared" si="0"/>
         <v>0.45045045045045046</v>
       </c>
-      <c r="J10" s="74"/>
-      <c r="K10" s="74"/>
-      <c r="L10" s="74"/>
+      <c r="J10" s="75"/>
+      <c r="K10" s="75"/>
+      <c r="L10" s="75"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="71">
+      <c r="A11" s="72">
         <v>46152</v>
       </c>
-      <c r="B11" s="72"/>
-      <c r="C11" s="72"/>
-      <c r="D11" s="72"/>
-      <c r="E11" s="73">
+      <c r="B11" s="73"/>
+      <c r="C11" s="73"/>
+      <c r="D11" s="73"/>
+      <c r="E11" s="74">
         <v>10.5</v>
       </c>
-      <c r="F11" s="73"/>
-      <c r="G11" s="73"/>
-      <c r="H11" s="73"/>
-      <c r="I11" s="74">
+      <c r="F11" s="74"/>
+      <c r="G11" s="74"/>
+      <c r="H11" s="74"/>
+      <c r="I11" s="75">
         <f t="shared" ref="I11" si="1">(E11-E10)/E10</f>
         <v>-0.86956521739130432</v>
       </c>
-      <c r="J11" s="74"/>
-      <c r="K11" s="74"/>
-      <c r="L11" s="74"/>
+      <c r="J11" s="75"/>
+      <c r="K11" s="75"/>
+      <c r="L11" s="75"/>
     </row>
   </sheetData>
   <mergeCells count="31">
@@ -5396,27 +5915,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="77" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="77" t="s">
+      <c r="C1" s="78" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77" t="s">
+      <c r="D1" s="78"/>
+      <c r="E1" s="78" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="77"/>
-      <c r="G1" s="76" t="s">
+      <c r="F1" s="78"/>
+      <c r="G1" s="77" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="76"/>
-      <c r="B2" s="76"/>
+      <c r="A2" s="77"/>
+      <c r="B2" s="77"/>
       <c r="C2" s="21" t="s">
         <v>33</v>
       </c>
@@ -5429,7 +5948,7 @@
       <c r="F2" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="76"/>
+      <c r="G2" s="77"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
@@ -5437,7 +5956,7 @@
       </c>
       <c r="B3" s="24">
         <f ca="1">RANDBETWEEN(10, 50)</f>
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C3" s="30">
         <f ca="1">RANDBETWEEN(2, 10)</f>
@@ -5445,19 +5964,19 @@
       </c>
       <c r="D3" s="22">
         <f ca="1">RANDBETWEEN(2, 10)</f>
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E3" s="29">
         <f ca="1">$B3*C3</f>
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="F3" s="35">
         <f ca="1">$B3*D3</f>
-        <v>120</v>
+        <v>38</v>
       </c>
       <c r="G3" s="38">
         <f ca="1">(E3+F3)/(E$8+F$8)</f>
-        <v>9.6106456382454408E-2</v>
+        <v>0.13768115942028986</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -5466,27 +5985,27 @@
       </c>
       <c r="B4" s="24">
         <f t="shared" ref="B4:B7" ca="1" si="0">RANDBETWEEN(10, 50)</f>
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="C4" s="31">
         <f t="shared" ref="C4:D7" ca="1" si="1">RANDBETWEEN(2, 10)</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D4" s="25">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4" s="29">
         <f t="shared" ref="E4:F7" ca="1" si="2">$B4*C4</f>
-        <v>280</v>
+        <v>115</v>
       </c>
       <c r="F4" s="36">
         <f t="shared" ca="1" si="2"/>
-        <v>120</v>
+        <v>46</v>
       </c>
       <c r="G4" s="38">
         <f ca="1">(E4+F4)/(E$8+F$8)</f>
-        <v>0.19714144898965008</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -5495,27 +6014,27 @@
       </c>
       <c r="B5" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="C5" s="31">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D5" s="28">
         <f t="shared" ca="1" si="1"/>
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E5" s="29">
         <f t="shared" ca="1" si="2"/>
-        <v>245</v>
+        <v>33</v>
       </c>
       <c r="F5" s="35">
         <f t="shared" ca="1" si="2"/>
-        <v>490</v>
+        <v>44</v>
       </c>
       <c r="G5" s="38">
         <f t="shared" ref="G5:G7" ca="1" si="3">(E5+F5)/(E$8+F$8)</f>
-        <v>0.36224741251848203</v>
+        <v>7.9710144927536225E-2</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -5524,27 +6043,27 @@
       </c>
       <c r="B6" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="C6" s="26">
         <f t="shared" ca="1" si="1"/>
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D6" s="25">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" s="29">
         <f t="shared" ca="1" si="2"/>
-        <v>333</v>
+        <v>69</v>
       </c>
       <c r="F6" s="35">
         <f t="shared" ca="1" si="2"/>
-        <v>111</v>
+        <v>46</v>
       </c>
       <c r="G6" s="38">
         <f t="shared" ca="1" si="3"/>
-        <v>0.21882700837851157</v>
+        <v>0.11904761904761904</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -5553,11 +6072,11 @@
       </c>
       <c r="B7" s="33">
         <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="C7" s="32">
         <f t="shared" ca="1" si="1"/>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D7" s="27">
         <f t="shared" ca="1" si="1"/>
@@ -5565,15 +6084,15 @@
       </c>
       <c r="E7" s="29">
         <f t="shared" ca="1" si="2"/>
-        <v>119</v>
+        <v>160</v>
       </c>
       <c r="F7" s="35">
         <f t="shared" ca="1" si="2"/>
-        <v>136</v>
+        <v>320</v>
       </c>
       <c r="G7" s="38">
         <f t="shared" ca="1" si="3"/>
-        <v>0.12567767373090191</v>
+        <v>0.49689440993788819</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -5585,11 +6104,11 @@
       <c r="D8" s="34"/>
       <c r="E8" s="37">
         <f ca="1">SUM(E3:E7)</f>
-        <v>1052</v>
+        <v>472</v>
       </c>
       <c r="F8" s="37">
         <f ca="1">SUM(F3:F7)</f>
-        <v>977</v>
+        <v>494</v>
       </c>
       <c r="G8" s="34"/>
     </row>
@@ -5627,10 +6146,10 @@
       <c r="C1" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="78" t="s">
+      <c r="F1" s="79" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="78"/>
+      <c r="G1" s="79"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="51" t="s">
@@ -5641,14 +6160,14 @@
       </c>
       <c r="C2" s="41">
         <f ca="1">RANDBETWEEN(500, 1000)</f>
-        <v>565</v>
+        <v>624</v>
       </c>
       <c r="F2" s="45" t="s">
         <v>48</v>
       </c>
       <c r="G2" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F2, $C$2:$C$9)</f>
-        <v>1061</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -5660,14 +6179,14 @@
       </c>
       <c r="C3" s="44">
         <f t="shared" ref="C3:C9" ca="1" si="0">RANDBETWEEN(500, 1000)</f>
-        <v>961</v>
+        <v>551</v>
       </c>
       <c r="F3" s="34" t="s">
         <v>50</v>
       </c>
       <c r="G3" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F3)</f>
-        <v>513</v>
+        <v>595</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -5679,14 +6198,14 @@
       </c>
       <c r="C4" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>630</v>
+        <v>902</v>
       </c>
       <c r="F4" s="34" t="s">
         <v>51</v>
       </c>
       <c r="G4" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F4)</f>
-        <v>548</v>
+        <v>860</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -5698,14 +6217,14 @@
       </c>
       <c r="C5" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>694</v>
+        <v>705</v>
       </c>
       <c r="F5" s="45" t="s">
         <v>46</v>
       </c>
       <c r="G5" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F5, $C$2:$C$9)</f>
-        <v>1526</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -5717,14 +6236,14 @@
       </c>
       <c r="C6" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>513</v>
+        <v>595</v>
       </c>
       <c r="F6" s="34" t="s">
         <v>50</v>
       </c>
       <c r="G6" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F6)</f>
-        <v>565</v>
+        <v>624</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -5736,14 +6255,14 @@
       </c>
       <c r="C7" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>548</v>
+        <v>860</v>
       </c>
       <c r="F7" s="34" t="s">
         <v>51</v>
       </c>
       <c r="G7" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F7)</f>
-        <v>961</v>
+        <v>551</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -5755,14 +6274,14 @@
       </c>
       <c r="C8" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>926</v>
+        <v>530</v>
       </c>
       <c r="F8" s="45" t="s">
         <v>47</v>
       </c>
       <c r="G8" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F8, $C$2:$C$9)</f>
-        <v>1324</v>
+        <v>1607</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -5774,14 +6293,14 @@
       </c>
       <c r="C9" s="42">
         <f t="shared" ca="1" si="0"/>
-        <v>613</v>
+        <v>902</v>
       </c>
       <c r="F9" s="34" t="s">
         <v>50</v>
       </c>
       <c r="G9" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F9)</f>
-        <v>630</v>
+        <v>902</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -5790,7 +6309,7 @@
       </c>
       <c r="G10" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F10)</f>
-        <v>694</v>
+        <v>705</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -5799,7 +6318,7 @@
       </c>
       <c r="G11" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F11, $C$2:$C$9)</f>
-        <v>1539</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -5808,7 +6327,7 @@
       </c>
       <c r="G12" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F12)</f>
-        <v>926</v>
+        <v>530</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -5817,7 +6336,7 @@
       </c>
       <c r="G13" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F13)</f>
-        <v>613</v>
+        <v>902</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -5826,7 +6345,7 @@
       </c>
       <c r="G14" s="43">
         <f ca="1">SUM(G2,G5,G8,G11)</f>
-        <v>5450</v>
+        <v>5669</v>
       </c>
     </row>
   </sheetData>
@@ -6011,10 +6530,10 @@
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C12" s="79" t="s">
+      <c r="C12" s="80" t="s">
         <v>74</v>
       </c>
-      <c r="D12" s="79"/>
+      <c r="D12" s="80"/>
       <c r="E12" s="66">
         <f>SUM(JLoka_Investors[INVESTMENT AMOUNT (USD)])</f>
         <v>180500</v>
@@ -6053,12 +6572,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B2" s="80" t="s">
+      <c r="B2" s="81" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
       <c r="F2" s="67"/>
     </row>
     <row r="3" spans="2:6" s="67" customFormat="1" x14ac:dyDescent="0.25">
@@ -6081,15 +6600,15 @@
       </c>
       <c r="C4" s="3">
         <f ca="1">RAND()</f>
-        <v>0.82725387354161772</v>
+        <v>0.1970140427985092</v>
       </c>
       <c r="D4" s="3">
         <f t="shared" ref="D4:E4" ca="1" si="0">RAND()</f>
-        <v>0.80017116372062791</v>
+        <v>0.61752950258084438</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.20801938180659352</v>
+        <v>0.59433522503123093</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -6098,15 +6617,15 @@
       </c>
       <c r="C5" s="3">
         <f t="shared" ref="C5:E14" ca="1" si="1">RAND()</f>
-        <v>0.98231634059209239</v>
+        <v>0.6633830799647159</v>
       </c>
       <c r="D5" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59857569406591837</v>
+        <v>0.52714726800078981</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>5.8172409636129241E-2</v>
+        <v>0.69668174009225037</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
@@ -6115,15 +6634,15 @@
       </c>
       <c r="C6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.92177328897518906</v>
+        <v>0.17562438708328187</v>
       </c>
       <c r="D6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.62960068734179109</v>
+        <v>0.9163764591219179</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.47613209032723569</v>
+        <v>0.98052310491075534</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
@@ -6132,15 +6651,15 @@
       </c>
       <c r="C7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>6.8127943760001086E-2</v>
+        <v>0.97179011742401034</v>
       </c>
       <c r="D7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.91148131598852689</v>
+        <v>0.86700995900552902</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.33943465465660472</v>
+        <v>0.53703235256206727</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
@@ -6149,15 +6668,15 @@
       </c>
       <c r="C8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.36546159306277792</v>
+        <v>0.84749572115146177</v>
       </c>
       <c r="D8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.49768864602230933</v>
+        <v>0.14018279942935719</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.56689538950625051</v>
+        <v>0.16890054256540799</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
@@ -6166,15 +6685,15 @@
       </c>
       <c r="C9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>7.0132702277079795E-2</v>
+        <v>0.93566798383572247</v>
       </c>
       <c r="D9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.39161580424131404</v>
+        <v>0.92855436625288845</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.70946690247282718</v>
+        <v>0.1460052583933078</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
@@ -6183,15 +6702,15 @@
       </c>
       <c r="C10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.29363415525332215</v>
+        <v>0.1433999468745274</v>
       </c>
       <c r="D10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3.4430219338273838E-2</v>
+        <v>0.63410830731845791</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.48517707387830089</v>
+        <v>0.6021723468059248</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
@@ -6200,15 +6719,15 @@
       </c>
       <c r="C11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.57614710490615306</v>
+        <v>0.21221459352036331</v>
       </c>
       <c r="D11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.88951744204066985</v>
+        <v>0.30477536836824548</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.34191490610491293</v>
+        <v>5.9313688358269889E-2</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
@@ -6217,15 +6736,15 @@
       </c>
       <c r="C12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.42653486070031332</v>
+        <v>4.7972957196397492E-2</v>
       </c>
       <c r="D12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.21054797943785342</v>
+        <v>0.63336008174203462</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.75340815882757395</v>
+        <v>0.19399467707450213</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
@@ -6234,15 +6753,15 @@
       </c>
       <c r="C13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.27532486384594812</v>
+        <v>0.72753524488705212</v>
       </c>
       <c r="D13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.29914873161213729</v>
+        <v>0.44769928553516947</v>
       </c>
       <c r="E13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.73473476496323886</v>
+        <v>0.22340416548027076</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
@@ -6251,15 +6770,15 @@
       </c>
       <c r="C14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.39228657162766789</v>
+        <v>0.89667820846322988</v>
       </c>
       <c r="D14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.72402950173284431</v>
+        <v>0.3584885461089784</v>
       </c>
       <c r="E14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>6.5175240099631937E-3</v>
+        <v>6.1928356350029135E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding the Finance sample
</commit_message>
<xml_diff>
--- a/Excel-Finance/JLoka-Finance-01.xlsx
+++ b/Excel-Finance/JLoka-Finance-01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\j-l-data-science-data-analytics\Excel-Finance\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\books-and-tutorials\Finance-Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602BA44E-F45F-417D-8C06-199DBCCCD0FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5CD25C-ECEB-425B-AB6B-644F84EF1AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="4" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="5" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,8 @@
     <sheet name="Sheet10" sheetId="10" r:id="rId10"/>
     <sheet name="Sheet11" sheetId="11" r:id="rId11"/>
     <sheet name="With XLOOKUP" sheetId="12" r:id="rId12"/>
+    <sheet name="Sheet12" sheetId="13" r:id="rId13"/>
+    <sheet name="Sheet13" sheetId="14" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet7!$B$1:$F$9</definedName>
@@ -38,8 +40,8 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicerCache r:id="rId13"/>
-        <x14:slicerCache r:id="rId14"/>
+        <x14:slicerCache r:id="rId15"/>
+        <x14:slicerCache r:id="rId16"/>
       </x15:slicerCaches>
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -58,8 +60,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="137">
   <si>
     <t>Sunday</t>
   </si>
@@ -407,6 +431,69 @@
   </si>
   <si>
     <t>Jloka-109</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Stock A</t>
+  </si>
+  <si>
+    <t>Stock B</t>
+  </si>
+  <si>
+    <t>Stock C</t>
+  </si>
+  <si>
+    <t>Index X</t>
+  </si>
+  <si>
+    <t>Index Y</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Row #</t>
+  </si>
+  <si>
+    <t>Column #</t>
+  </si>
+  <si>
+    <t>Stock Ticker</t>
+  </si>
+  <si>
+    <t>Number Of Shares</t>
+  </si>
+  <si>
+    <t>Price Per Share</t>
+  </si>
+  <si>
+    <t>Total Value</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-05</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-06</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-07</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-08</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-09</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-10</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-11</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -465,7 +552,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,8 +625,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="26">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -872,13 +965,97 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -990,7 +1167,16 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1002,10 +1188,7 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1023,6 +1206,29 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1693,31 +1899,31 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.17562438708328187</c:v>
+                  <c:v>0.56155399528444627</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.97179011742401034</c:v>
+                  <c:v>0.52126929017846724</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.84749572115146177</c:v>
+                  <c:v>0.97925953918999264</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.93566798383572247</c:v>
+                  <c:v>0.10034826295175892</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.1433999468745274</c:v>
+                  <c:v>0.9503281952830277</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.21221459352036331</c:v>
+                  <c:v>0.87703057541907758</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.7972957196397492E-2</c:v>
+                  <c:v>0.80006013547308241</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.72753524488705212</c:v>
+                  <c:v>0.28464794699125118</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.89667820846322988</c:v>
+                  <c:v>0.29989699726608532</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1857,31 +2063,31 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.9163764591219179</c:v>
+                  <c:v>0.68186447037085673</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.86700995900552902</c:v>
+                  <c:v>0.60875095923928202</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.14018279942935719</c:v>
+                  <c:v>0.88291092579954622</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.92855436625288845</c:v>
+                  <c:v>0.58665416372055923</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.63410830731845791</c:v>
+                  <c:v>0.33359262369764586</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.30477536836824548</c:v>
+                  <c:v>0.80630794943668815</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.63336008174203462</c:v>
+                  <c:v>0.52751584656207184</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.44769928553516947</c:v>
+                  <c:v>0.39156857781522625</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.3584885461089784</c:v>
+                  <c:v>0.19502874159617778</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2021,31 +2227,31 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.98052310491075534</c:v>
+                  <c:v>0.22676712201392224</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.53703235256206727</c:v>
+                  <c:v>0.84204372880442302</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.16890054256540799</c:v>
+                  <c:v>0.45790128096059224</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1460052583933078</c:v>
+                  <c:v>0.36038891406072593</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.6021723468059248</c:v>
+                  <c:v>0.75719536474901727</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.9313688358269889E-2</c:v>
+                  <c:v>0.15921596559988871</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.19399467707450213</c:v>
+                  <c:v>0.92639734750661817</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.22340416548027076</c:v>
+                  <c:v>0.52483943302404878</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6.1928356350029135E-2</c:v>
+                  <c:v>0.57672047294585982</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4816,22 +5022,22 @@
       </c>
       <c r="D3" s="2">
         <f ca="1">RANDBETWEEN(250, 3200)</f>
-        <v>1889</v>
+        <v>1106</v>
       </c>
       <c r="E3" s="70">
         <f ca="1">RANDBETWEEN(0, 2)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G3" t="s">
         <v>77</v>
       </c>
       <c r="H3" s="2">
         <f ca="1">VLOOKUP($G3, Table1[], 3, FALSE)</f>
-        <v>1889</v>
+        <v>1106</v>
       </c>
       <c r="I3" s="2">
         <f ca="1">VLOOKUP($G3, Table1[], 4, FALSE)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
@@ -4843,7 +5049,7 @@
       </c>
       <c r="D4" s="2">
         <f t="shared" ref="D4:D12" ca="1" si="0">RANDBETWEEN(250, 3200)</f>
-        <v>2579</v>
+        <v>1747</v>
       </c>
       <c r="E4" s="70">
         <f t="shared" ref="E4:E12" ca="1" si="1">RANDBETWEEN(0, 2)</f>
@@ -4854,7 +5060,7 @@
       </c>
       <c r="H4" s="2">
         <f ca="1">VLOOKUP($G4, Table1[], 3, FALSE)</f>
-        <v>2579</v>
+        <v>1747</v>
       </c>
       <c r="I4" s="2">
         <f ca="1">VLOOKUP($G4, Table1[], 4, FALSE)</f>
@@ -4870,22 +5076,22 @@
       </c>
       <c r="D5" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>2328</v>
+        <v>690</v>
       </c>
       <c r="E5" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" t="s">
         <v>79</v>
       </c>
       <c r="H5" s="2">
         <f ca="1">VLOOKUP($G5, Table1[], 3, FALSE)</f>
-        <v>3058</v>
+        <v>769</v>
       </c>
       <c r="I5" s="2">
         <f ca="1">VLOOKUP($G5, Table1[], 4, FALSE)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
@@ -4897,18 +5103,18 @@
       </c>
       <c r="D6" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>1742</v>
+        <v>1970</v>
       </c>
       <c r="E6" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G6" t="s">
         <v>105</v>
       </c>
       <c r="H6" s="2">
         <f ca="1">VLOOKUP($G6, Table1[], 3, FALSE)</f>
-        <v>1368</v>
+        <v>2844</v>
       </c>
       <c r="I6" s="2">
         <f ca="1">VLOOKUP($G6, Table1[], 4, FALSE)</f>
@@ -4924,7 +5130,7 @@
       </c>
       <c r="D7" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>2717</v>
+        <v>2084</v>
       </c>
       <c r="E7" s="70">
         <f t="shared" ca="1" si="1"/>
@@ -4940,11 +5146,11 @@
       </c>
       <c r="D8" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>3058</v>
+        <v>769</v>
       </c>
       <c r="E8" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
@@ -4956,11 +5162,11 @@
       </c>
       <c r="D9" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>2576</v>
+        <v>1694</v>
       </c>
       <c r="E9" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
@@ -4972,11 +5178,11 @@
       </c>
       <c r="D10" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>2568</v>
+        <v>914</v>
       </c>
       <c r="E10" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
@@ -4988,7 +5194,7 @@
       </c>
       <c r="D11" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>1368</v>
+        <v>2844</v>
       </c>
       <c r="E11" s="70">
         <f t="shared" ca="1" si="1"/>
@@ -5004,11 +5210,11 @@
       </c>
       <c r="D12" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>2086</v>
+        <v>302</v>
       </c>
       <c r="E12" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5067,7 +5273,7 @@
       </c>
       <c r="D3" s="2">
         <f ca="1">RANDBETWEEN(250, 3200)</f>
-        <v>607</v>
+        <v>1397</v>
       </c>
       <c r="E3" s="70">
         <f ca="1">RANDBETWEEN(0, 2)</f>
@@ -5078,7 +5284,7 @@
       </c>
       <c r="H3" s="2">
         <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Price], "Missing")</f>
-        <v>607</v>
+        <v>1397</v>
       </c>
       <c r="I3" s="2">
         <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Dividend], "Missing")</f>
@@ -5094,22 +5300,22 @@
       </c>
       <c r="D4" s="2">
         <f t="shared" ref="D4:D12" ca="1" si="0">RANDBETWEEN(250, 3200)</f>
-        <v>2613</v>
+        <v>775</v>
       </c>
       <c r="E4" s="70">
         <f t="shared" ref="E4:E12" ca="1" si="1">RANDBETWEEN(0, 2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="s">
         <v>78</v>
       </c>
       <c r="H4" s="2">
         <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Price], "Missing")</f>
-        <v>2613</v>
+        <v>775</v>
       </c>
       <c r="I4" s="2">
         <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Dividend], "Missing")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
@@ -5121,22 +5327,22 @@
       </c>
       <c r="D5" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>769</v>
+        <v>1215</v>
       </c>
       <c r="E5" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" t="s">
         <v>79</v>
       </c>
       <c r="H5" s="2">
         <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Price], "Missing")</f>
-        <v>732</v>
+        <v>374</v>
       </c>
       <c r="I5" s="2">
         <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Dividend], "Missing")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
@@ -5148,18 +5354,18 @@
       </c>
       <c r="D6" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>816</v>
+        <v>2092</v>
       </c>
       <c r="E6" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="s">
         <v>105</v>
       </c>
       <c r="H6" s="2">
         <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Price], "Missing")</f>
-        <v>3071</v>
+        <v>838</v>
       </c>
       <c r="I6" s="2">
         <f ca="1">_xlfn.XLOOKUP(Table69[[#This Row],[Ticker]], Table18[Ticker], Table18[Dividend], "Missing")</f>
@@ -5175,7 +5381,7 @@
       </c>
       <c r="D7" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>1890</v>
+        <v>2163</v>
       </c>
       <c r="E7" s="70">
         <f t="shared" ca="1" si="1"/>
@@ -5191,11 +5397,11 @@
       </c>
       <c r="D8" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>732</v>
+        <v>374</v>
       </c>
       <c r="E8" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
@@ -5207,7 +5413,7 @@
       </c>
       <c r="D9" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>3200</v>
+        <v>253</v>
       </c>
       <c r="E9" s="70">
         <f t="shared" ca="1" si="1"/>
@@ -5223,11 +5429,11 @@
       </c>
       <c r="D10" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>2186</v>
+        <v>631</v>
       </c>
       <c r="E10" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
@@ -5239,7 +5445,7 @@
       </c>
       <c r="D11" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>3071</v>
+        <v>838</v>
       </c>
       <c r="E11" s="70">
         <f t="shared" ca="1" si="1"/>
@@ -5255,11 +5461,11 @@
       </c>
       <c r="D12" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>1931</v>
+        <v>864</v>
       </c>
       <c r="E12" s="70">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5268,6 +5474,511 @@
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
   </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EC1371C-14AF-4334-8E19-C4A01FA044F1}">
+  <dimension ref="B2:M8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.140625" customWidth="1"/>
+    <col min="13" max="13" width="26.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B2" s="84" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" s="84" t="s">
+        <v>117</v>
+      </c>
+      <c r="D2" s="84" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" s="84" t="s">
+        <v>119</v>
+      </c>
+      <c r="F2" s="84" t="s">
+        <v>120</v>
+      </c>
+      <c r="G2" s="84" t="s">
+        <v>121</v>
+      </c>
+      <c r="I2" s="85" t="s">
+        <v>116</v>
+      </c>
+      <c r="J2" s="85" t="s">
+        <v>122</v>
+      </c>
+      <c r="K2" s="85" t="s">
+        <v>123</v>
+      </c>
+      <c r="L2" s="85" t="s">
+        <v>124</v>
+      </c>
+      <c r="M2" s="85" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B3" s="86">
+        <v>46045</v>
+      </c>
+      <c r="C3" s="72">
+        <f ca="1">RANDBETWEEN(120, 150)</f>
+        <v>135</v>
+      </c>
+      <c r="D3" s="72">
+        <f ca="1">RANDBETWEEN(210, 260)</f>
+        <v>259</v>
+      </c>
+      <c r="E3" s="72">
+        <f ca="1">RANDBETWEEN(330, 380)</f>
+        <v>342</v>
+      </c>
+      <c r="F3" s="72">
+        <v>1250</v>
+      </c>
+      <c r="G3" s="72">
+        <v>2350</v>
+      </c>
+      <c r="I3" s="86">
+        <v>46076</v>
+      </c>
+      <c r="J3" s="71" t="s">
+        <v>119</v>
+      </c>
+      <c r="K3" s="71">
+        <f>MATCH(I3, $B$3:$B$8,0)</f>
+        <v>2</v>
+      </c>
+      <c r="L3" s="71">
+        <f>MATCH(J3,$C$2:$G$2,0)</f>
+        <v>3</v>
+      </c>
+      <c r="M3" s="72" cm="1">
+        <f t="array" aca="1" ref="M3" ca="1">INDEX($C$3:$G$8, K3,L3)</f>
+        <v>343</v>
+      </c>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B4" s="86">
+        <v>46076</v>
+      </c>
+      <c r="C4" s="72">
+        <f t="shared" ref="C4:C8" ca="1" si="0">RANDBETWEEN(120, 150)</f>
+        <v>148</v>
+      </c>
+      <c r="D4" s="72">
+        <f t="shared" ref="D4:D8" ca="1" si="1">RANDBETWEEN(210, 260)</f>
+        <v>231</v>
+      </c>
+      <c r="E4" s="72">
+        <f t="shared" ref="E4:E8" ca="1" si="2">RANDBETWEEN(330, 380)</f>
+        <v>343</v>
+      </c>
+      <c r="F4" s="72">
+        <v>1300</v>
+      </c>
+      <c r="G4" s="72">
+        <v>2400</v>
+      </c>
+      <c r="I4" s="86">
+        <v>46076</v>
+      </c>
+      <c r="J4" s="71" t="s">
+        <v>118</v>
+      </c>
+      <c r="K4" s="71">
+        <f t="shared" ref="K4:K7" si="3">MATCH(I4, $B$3:$B$8,0)</f>
+        <v>2</v>
+      </c>
+      <c r="L4" s="71">
+        <f t="shared" ref="L4:L7" si="4">MATCH(J4,$C$2:$G$2,0)</f>
+        <v>2</v>
+      </c>
+      <c r="M4" s="72" cm="1">
+        <f t="array" aca="1" ref="M4" ca="1">INDEX($C$3:$G$8, K4,L4)</f>
+        <v>231</v>
+      </c>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B5" s="86">
+        <v>46104</v>
+      </c>
+      <c r="C5" s="72">
+        <f t="shared" ca="1" si="0"/>
+        <v>124</v>
+      </c>
+      <c r="D5" s="72">
+        <f t="shared" ca="1" si="1"/>
+        <v>246</v>
+      </c>
+      <c r="E5" s="72">
+        <f t="shared" ca="1" si="2"/>
+        <v>341</v>
+      </c>
+      <c r="F5" s="72">
+        <v>1350</v>
+      </c>
+      <c r="G5" s="72">
+        <v>2450</v>
+      </c>
+      <c r="I5" s="86">
+        <v>46104</v>
+      </c>
+      <c r="J5" s="71" t="s">
+        <v>120</v>
+      </c>
+      <c r="K5" s="71">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="L5" s="71">
+        <f t="shared" si="4"/>
+        <v>4</v>
+      </c>
+      <c r="M5" s="72" cm="1">
+        <f t="array" ref="M5">INDEX($C$3:$G$8, K5,L5)</f>
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B6" s="86">
+        <v>46135</v>
+      </c>
+      <c r="C6" s="72">
+        <f t="shared" ca="1" si="0"/>
+        <v>128</v>
+      </c>
+      <c r="D6" s="72">
+        <f t="shared" ca="1" si="1"/>
+        <v>217</v>
+      </c>
+      <c r="E6" s="72">
+        <f t="shared" ca="1" si="2"/>
+        <v>343</v>
+      </c>
+      <c r="F6" s="72">
+        <v>1400</v>
+      </c>
+      <c r="G6" s="72">
+        <v>2500</v>
+      </c>
+      <c r="I6" s="86">
+        <v>46135</v>
+      </c>
+      <c r="J6" s="71" t="s">
+        <v>120</v>
+      </c>
+      <c r="K6" s="71">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="L6" s="71">
+        <f t="shared" si="4"/>
+        <v>4</v>
+      </c>
+      <c r="M6" s="72" cm="1">
+        <f t="array" ref="M6">INDEX($C$3:$G$8, K6,L6)</f>
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B7" s="86">
+        <v>46165</v>
+      </c>
+      <c r="C7" s="72">
+        <f t="shared" ca="1" si="0"/>
+        <v>123</v>
+      </c>
+      <c r="D7" s="72">
+        <f t="shared" ca="1" si="1"/>
+        <v>212</v>
+      </c>
+      <c r="E7" s="72">
+        <f t="shared" ca="1" si="2"/>
+        <v>361</v>
+      </c>
+      <c r="F7" s="72">
+        <v>1450</v>
+      </c>
+      <c r="G7" s="72">
+        <v>2550</v>
+      </c>
+      <c r="I7" s="86">
+        <v>46196</v>
+      </c>
+      <c r="J7" s="71" t="s">
+        <v>121</v>
+      </c>
+      <c r="K7" s="71">
+        <f t="shared" si="3"/>
+        <v>6</v>
+      </c>
+      <c r="L7" s="71">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="M7" s="72" cm="1">
+        <f t="array" ref="M7">INDEX($C$3:$G$8, K7,L7)</f>
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B8" s="86">
+        <v>46196</v>
+      </c>
+      <c r="C8" s="72">
+        <f t="shared" ca="1" si="0"/>
+        <v>123</v>
+      </c>
+      <c r="D8" s="72">
+        <f t="shared" ca="1" si="1"/>
+        <v>257</v>
+      </c>
+      <c r="E8" s="72">
+        <f t="shared" ca="1" si="2"/>
+        <v>376</v>
+      </c>
+      <c r="F8" s="72">
+        <v>1500</v>
+      </c>
+      <c r="G8" s="72">
+        <v>2600</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FAAC275-79FD-4ECC-93CD-B834A0A54184}">
+  <dimension ref="B2:E14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="87" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="88" t="s">
+        <v>126</v>
+      </c>
+      <c r="D2" s="88" t="s">
+        <v>127</v>
+      </c>
+      <c r="E2" s="89" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="90">
+        <f ca="1">RANDBETWEEN(5, 50)</f>
+        <v>11</v>
+      </c>
+      <c r="D3" s="91">
+        <f ca="1">RANDBETWEEN(1000, 100000)</f>
+        <v>37172</v>
+      </c>
+      <c r="E3" s="98" cm="1">
+        <f t="array" aca="1" ref="E3:E13" ca="1">C3:C13*D3:D13</f>
+        <v>408892</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="90">
+        <f t="shared" ref="C4:C13" ca="1" si="0">RANDBETWEEN(5, 50)</f>
+        <v>20</v>
+      </c>
+      <c r="D4" s="91">
+        <f t="shared" ref="D4:D13" ca="1" si="1">RANDBETWEEN(1000, 100000)</f>
+        <v>23333</v>
+      </c>
+      <c r="E4" s="99">
+        <f ca="1"/>
+        <v>466660</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="90">
+        <f t="shared" ca="1" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="D5" s="91">
+        <f t="shared" ca="1" si="1"/>
+        <v>6539</v>
+      </c>
+      <c r="E5" s="99">
+        <f ca="1"/>
+        <v>170014</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="90">
+        <f t="shared" ca="1" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="D6" s="91">
+        <f t="shared" ca="1" si="1"/>
+        <v>49878</v>
+      </c>
+      <c r="E6" s="99">
+        <f ca="1"/>
+        <v>1745730</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="32" t="s">
+        <v>129</v>
+      </c>
+      <c r="C7" s="90">
+        <f t="shared" ca="1" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="D7" s="91">
+        <f t="shared" ca="1" si="1"/>
+        <v>36062</v>
+      </c>
+      <c r="E7" s="99">
+        <f ca="1"/>
+        <v>937612</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="32" t="s">
+        <v>130</v>
+      </c>
+      <c r="C8" s="90">
+        <f t="shared" ca="1" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="D8" s="91">
+        <f t="shared" ca="1" si="1"/>
+        <v>65797</v>
+      </c>
+      <c r="E8" s="99">
+        <f ca="1"/>
+        <v>2763474</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="32" t="s">
+        <v>131</v>
+      </c>
+      <c r="C9" s="90">
+        <f t="shared" ca="1" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="D9" s="91">
+        <f t="shared" ca="1" si="1"/>
+        <v>64179</v>
+      </c>
+      <c r="E9" s="99">
+        <f ca="1"/>
+        <v>1155222</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="32" t="s">
+        <v>132</v>
+      </c>
+      <c r="C10" s="90">
+        <f t="shared" ca="1" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="D10" s="91">
+        <f t="shared" ca="1" si="1"/>
+        <v>8015</v>
+      </c>
+      <c r="E10" s="99">
+        <f ca="1"/>
+        <v>192360</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="32" t="s">
+        <v>133</v>
+      </c>
+      <c r="C11" s="90">
+        <f t="shared" ca="1" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="D11" s="91">
+        <f t="shared" ca="1" si="1"/>
+        <v>18216</v>
+      </c>
+      <c r="E11" s="99">
+        <f ca="1"/>
+        <v>218592</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="32" t="s">
+        <v>134</v>
+      </c>
+      <c r="C12" s="90">
+        <f t="shared" ca="1" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="D12" s="91">
+        <f t="shared" ca="1" si="1"/>
+        <v>87309</v>
+      </c>
+      <c r="E12" s="99">
+        <f ca="1"/>
+        <v>960399</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="92" t="s">
+        <v>135</v>
+      </c>
+      <c r="C13" s="93">
+        <f t="shared" ca="1" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="D13" s="94">
+        <f t="shared" ca="1" si="1"/>
+        <v>39167</v>
+      </c>
+      <c r="E13" s="100">
+        <f ca="1"/>
+        <v>509171</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="95" t="s">
+        <v>136</v>
+      </c>
+      <c r="C14" s="96"/>
+      <c r="D14" s="96"/>
+      <c r="E14" s="97"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -5367,243 +6078,258 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="74" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
+      <c r="I1" s="74"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="74"/>
+      <c r="L1" s="74"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="78" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71" t="s">
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71" t="s">
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="71"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="72">
+      <c r="A3" s="75">
         <v>46144</v>
       </c>
-      <c r="B3" s="73"/>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
-      <c r="E3" s="74">
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="77">
         <v>250.25</v>
       </c>
-      <c r="F3" s="74"/>
-      <c r="G3" s="74"/>
-      <c r="H3" s="74"/>
-      <c r="I3" s="73"/>
-      <c r="J3" s="73"/>
-      <c r="K3" s="73"/>
-      <c r="L3" s="73"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="76"/>
+      <c r="L3" s="76"/>
       <c r="N3" s="11" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="72">
+      <c r="A4" s="75">
         <v>46145</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="74">
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="77">
         <v>300</v>
       </c>
-      <c r="F4" s="74"/>
-      <c r="G4" s="74"/>
-      <c r="H4" s="74"/>
-      <c r="I4" s="75">
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
+      <c r="I4" s="73">
         <f>(E4-E3)/E3</f>
         <v>0.19880119880119881</v>
       </c>
-      <c r="J4" s="75"/>
-      <c r="K4" s="75"/>
-      <c r="L4" s="75"/>
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
+      <c r="L4" s="73"/>
       <c r="N4" s="10">
         <f>AVERAGE(I4:L11)</f>
         <v>-8.1596436336491718E-2</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="72">
+      <c r="A5" s="75">
         <v>46146</v>
       </c>
-      <c r="B5" s="73"/>
-      <c r="C5" s="73"/>
-      <c r="D5" s="73"/>
-      <c r="E5" s="74">
+      <c r="B5" s="76"/>
+      <c r="C5" s="76"/>
+      <c r="D5" s="76"/>
+      <c r="E5" s="77">
         <v>350.15</v>
       </c>
-      <c r="F5" s="74"/>
-      <c r="G5" s="74"/>
-      <c r="H5" s="74"/>
-      <c r="I5" s="75">
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="77"/>
+      <c r="I5" s="73">
         <f>(E5-E4)/E4</f>
         <v>0.1671666666666666</v>
       </c>
-      <c r="J5" s="75"/>
-      <c r="K5" s="75"/>
-      <c r="L5" s="75"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="73"/>
+      <c r="L5" s="73"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="72">
+      <c r="A6" s="75">
         <v>46147</v>
       </c>
-      <c r="B6" s="73"/>
-      <c r="C6" s="73"/>
-      <c r="D6" s="73"/>
-      <c r="E6" s="74">
+      <c r="B6" s="76"/>
+      <c r="C6" s="76"/>
+      <c r="D6" s="76"/>
+      <c r="E6" s="77">
         <v>650.5</v>
       </c>
-      <c r="F6" s="74"/>
-      <c r="G6" s="74"/>
-      <c r="H6" s="74"/>
-      <c r="I6" s="75">
+      <c r="F6" s="77"/>
+      <c r="G6" s="77"/>
+      <c r="H6" s="77"/>
+      <c r="I6" s="73">
         <f>(E6-E5)/E5</f>
         <v>0.85777523918320731</v>
       </c>
-      <c r="J6" s="75"/>
-      <c r="K6" s="75"/>
-      <c r="L6" s="75"/>
+      <c r="J6" s="73"/>
+      <c r="K6" s="73"/>
+      <c r="L6" s="73"/>
       <c r="N6" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="72">
+      <c r="A7" s="75">
         <v>46148</v>
       </c>
-      <c r="B7" s="73"/>
-      <c r="C7" s="73"/>
-      <c r="D7" s="73"/>
-      <c r="E7" s="74">
+      <c r="B7" s="76"/>
+      <c r="C7" s="76"/>
+      <c r="D7" s="76"/>
+      <c r="E7" s="77">
         <v>600.35</v>
       </c>
-      <c r="F7" s="74"/>
-      <c r="G7" s="74"/>
-      <c r="H7" s="74"/>
-      <c r="I7" s="75">
+      <c r="F7" s="77"/>
+      <c r="G7" s="77"/>
+      <c r="H7" s="77"/>
+      <c r="I7" s="73">
         <f t="shared" ref="I7:I10" si="0">(E7-E6)/E6</f>
         <v>-7.7094542659492657E-2</v>
       </c>
-      <c r="J7" s="75"/>
-      <c r="K7" s="75"/>
-      <c r="L7" s="75"/>
+      <c r="J7" s="73"/>
+      <c r="K7" s="73"/>
+      <c r="L7" s="73"/>
       <c r="N7" s="12" t="str">
         <f>IF(N4&gt;0,"Positive","Negative")</f>
         <v>Negative</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="72">
+      <c r="A8" s="75">
         <v>46149</v>
       </c>
-      <c r="B8" s="73"/>
-      <c r="C8" s="73"/>
-      <c r="D8" s="73"/>
-      <c r="E8" s="74">
+      <c r="B8" s="76"/>
+      <c r="C8" s="76"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="77">
         <v>150.19999999999999</v>
       </c>
-      <c r="F8" s="74"/>
-      <c r="G8" s="74"/>
-      <c r="H8" s="74"/>
-      <c r="I8" s="75">
+      <c r="F8" s="77"/>
+      <c r="G8" s="77"/>
+      <c r="H8" s="77"/>
+      <c r="I8" s="73">
         <f t="shared" si="0"/>
         <v>-0.74981260931123517</v>
       </c>
-      <c r="J8" s="75"/>
-      <c r="K8" s="75"/>
-      <c r="L8" s="75"/>
+      <c r="J8" s="73"/>
+      <c r="K8" s="73"/>
+      <c r="L8" s="73"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="72">
+      <c r="A9" s="75">
         <v>46150</v>
       </c>
-      <c r="B9" s="73"/>
-      <c r="C9" s="73"/>
-      <c r="D9" s="73"/>
-      <c r="E9" s="74">
+      <c r="B9" s="76"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="77">
         <v>55.5</v>
       </c>
-      <c r="F9" s="74"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="74"/>
-      <c r="I9" s="75">
+      <c r="F9" s="77"/>
+      <c r="G9" s="77"/>
+      <c r="H9" s="77"/>
+      <c r="I9" s="73">
         <f t="shared" si="0"/>
         <v>-0.6304926764314247</v>
       </c>
-      <c r="J9" s="75"/>
-      <c r="K9" s="75"/>
-      <c r="L9" s="75"/>
+      <c r="J9" s="73"/>
+      <c r="K9" s="73"/>
+      <c r="L9" s="73"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="72">
+      <c r="A10" s="75">
         <v>46151</v>
       </c>
-      <c r="B10" s="73"/>
-      <c r="C10" s="73"/>
-      <c r="D10" s="73"/>
-      <c r="E10" s="74">
+      <c r="B10" s="76"/>
+      <c r="C10" s="76"/>
+      <c r="D10" s="76"/>
+      <c r="E10" s="77">
         <v>80.5</v>
       </c>
-      <c r="F10" s="74"/>
-      <c r="G10" s="74"/>
-      <c r="H10" s="74"/>
-      <c r="I10" s="75">
+      <c r="F10" s="77"/>
+      <c r="G10" s="77"/>
+      <c r="H10" s="77"/>
+      <c r="I10" s="73">
         <f t="shared" si="0"/>
         <v>0.45045045045045046</v>
       </c>
-      <c r="J10" s="75"/>
-      <c r="K10" s="75"/>
-      <c r="L10" s="75"/>
+      <c r="J10" s="73"/>
+      <c r="K10" s="73"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="72">
+      <c r="A11" s="75">
         <v>46152</v>
       </c>
-      <c r="B11" s="73"/>
-      <c r="C11" s="73"/>
-      <c r="D11" s="73"/>
-      <c r="E11" s="74">
+      <c r="B11" s="76"/>
+      <c r="C11" s="76"/>
+      <c r="D11" s="76"/>
+      <c r="E11" s="77">
         <v>10.5</v>
       </c>
-      <c r="F11" s="74"/>
-      <c r="G11" s="74"/>
-      <c r="H11" s="74"/>
-      <c r="I11" s="75">
+      <c r="F11" s="77"/>
+      <c r="G11" s="77"/>
+      <c r="H11" s="77"/>
+      <c r="I11" s="73">
         <f t="shared" ref="I11" si="1">(E11-E10)/E10</f>
         <v>-0.86956521739130432</v>
       </c>
-      <c r="J11" s="75"/>
-      <c r="K11" s="75"/>
-      <c r="L11" s="75"/>
+      <c r="J11" s="73"/>
+      <c r="K11" s="73"/>
+      <c r="L11" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A7:D7"/>
     <mergeCell ref="I10:L10"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A11:D11"/>
@@ -5620,21 +6346,6 @@
     <mergeCell ref="I9:L9"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="E6:H6"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5915,27 +6626,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="79" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="77" t="s">
+      <c r="B1" s="79" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="78" t="s">
+      <c r="C1" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78" t="s">
+      <c r="D1" s="80"/>
+      <c r="E1" s="80" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="78"/>
-      <c r="G1" s="77" t="s">
+      <c r="F1" s="80"/>
+      <c r="G1" s="79" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="77"/>
-      <c r="B2" s="77"/>
+      <c r="A2" s="79"/>
+      <c r="B2" s="79"/>
       <c r="C2" s="21" t="s">
         <v>33</v>
       </c>
@@ -5948,7 +6659,7 @@
       <c r="F2" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="77"/>
+      <c r="G2" s="79"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
@@ -5956,27 +6667,27 @@
       </c>
       <c r="B3" s="24">
         <f ca="1">RANDBETWEEN(10, 50)</f>
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C3" s="30">
         <f ca="1">RANDBETWEEN(2, 10)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3" s="22">
         <f ca="1">RANDBETWEEN(2, 10)</f>
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E3" s="29">
         <f ca="1">$B3*C3</f>
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F3" s="35">
         <f ca="1">$B3*D3</f>
-        <v>38</v>
+        <v>91</v>
       </c>
       <c r="G3" s="38">
         <f ca="1">(E3+F3)/(E$8+F$8)</f>
-        <v>0.13768115942028986</v>
+        <v>0.12037037037037036</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -5985,27 +6696,27 @@
       </c>
       <c r="B4" s="24">
         <f t="shared" ref="B4:B7" ca="1" si="0">RANDBETWEEN(10, 50)</f>
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C4" s="31">
         <f t="shared" ref="C4:D7" ca="1" si="1">RANDBETWEEN(2, 10)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" s="25">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E4" s="29">
         <f t="shared" ref="E4:F7" ca="1" si="2">$B4*C4</f>
-        <v>115</v>
+        <v>40</v>
       </c>
       <c r="F4" s="36">
         <f t="shared" ca="1" si="2"/>
-        <v>46</v>
+        <v>90</v>
       </c>
       <c r="G4" s="38">
         <f ca="1">(E4+F4)/(E$8+F$8)</f>
-        <v>0.16666666666666666</v>
+        <v>8.5978835978835974E-2</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -6014,27 +6725,27 @@
       </c>
       <c r="B5" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="C5" s="31">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" s="28">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E5" s="29">
         <f t="shared" ca="1" si="2"/>
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="F5" s="35">
         <f t="shared" ca="1" si="2"/>
-        <v>44</v>
+        <v>336</v>
       </c>
       <c r="G5" s="38">
         <f t="shared" ref="G5:G7" ca="1" si="3">(E5+F5)/(E$8+F$8)</f>
-        <v>7.9710144927536225E-2</v>
+        <v>0.27777777777777779</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -6043,27 +6754,27 @@
       </c>
       <c r="B6" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C6" s="26">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" s="25">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E6" s="29">
         <f t="shared" ca="1" si="2"/>
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="F6" s="35">
         <f t="shared" ca="1" si="2"/>
-        <v>46</v>
+        <v>150</v>
       </c>
       <c r="G6" s="38">
         <f t="shared" ca="1" si="3"/>
-        <v>0.11904761904761904</v>
+        <v>0.13227513227513227</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -6072,27 +6783,27 @@
       </c>
       <c r="B7" s="33">
         <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="C7" s="32">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D7" s="27">
         <f t="shared" ca="1" si="1"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E7" s="29">
         <f t="shared" ca="1" si="2"/>
-        <v>160</v>
+        <v>290</v>
       </c>
       <c r="F7" s="35">
         <f t="shared" ca="1" si="2"/>
-        <v>320</v>
+        <v>290</v>
       </c>
       <c r="G7" s="38">
         <f t="shared" ca="1" si="3"/>
-        <v>0.49689440993788819</v>
+        <v>0.3835978835978836</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -6104,11 +6815,11 @@
       <c r="D8" s="34"/>
       <c r="E8" s="37">
         <f ca="1">SUM(E3:E7)</f>
-        <v>472</v>
+        <v>555</v>
       </c>
       <c r="F8" s="37">
         <f ca="1">SUM(F3:F7)</f>
-        <v>494</v>
+        <v>957</v>
       </c>
       <c r="G8" s="34"/>
     </row>
@@ -6146,10 +6857,10 @@
       <c r="C1" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="79" t="s">
+      <c r="F1" s="81" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="79"/>
+      <c r="G1" s="81"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="51" t="s">
@@ -6160,14 +6871,14 @@
       </c>
       <c r="C2" s="41">
         <f ca="1">RANDBETWEEN(500, 1000)</f>
-        <v>624</v>
+        <v>813</v>
       </c>
       <c r="F2" s="45" t="s">
         <v>48</v>
       </c>
       <c r="G2" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F2, $C$2:$C$9)</f>
-        <v>1455</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -6179,14 +6890,14 @@
       </c>
       <c r="C3" s="44">
         <f t="shared" ref="C3:C9" ca="1" si="0">RANDBETWEEN(500, 1000)</f>
-        <v>551</v>
+        <v>970</v>
       </c>
       <c r="F3" s="34" t="s">
         <v>50</v>
       </c>
       <c r="G3" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F3)</f>
-        <v>595</v>
+        <v>504</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -6198,14 +6909,14 @@
       </c>
       <c r="C4" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>902</v>
+        <v>960</v>
       </c>
       <c r="F4" s="34" t="s">
         <v>51</v>
       </c>
       <c r="G4" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F2, $B$2:$B$9, F4)</f>
-        <v>860</v>
+        <v>702</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -6217,14 +6928,14 @@
       </c>
       <c r="C5" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>705</v>
+        <v>822</v>
       </c>
       <c r="F5" s="45" t="s">
         <v>46</v>
       </c>
       <c r="G5" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F5, $C$2:$C$9)</f>
-        <v>1175</v>
+        <v>1783</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -6236,14 +6947,14 @@
       </c>
       <c r="C6" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>595</v>
+        <v>504</v>
       </c>
       <c r="F6" s="34" t="s">
         <v>50</v>
       </c>
       <c r="G6" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F6)</f>
-        <v>624</v>
+        <v>813</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -6255,14 +6966,14 @@
       </c>
       <c r="C7" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>860</v>
+        <v>702</v>
       </c>
       <c r="F7" s="34" t="s">
         <v>51</v>
       </c>
       <c r="G7" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F5, $B$2:$B$9, F7)</f>
-        <v>551</v>
+        <v>970</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -6274,14 +6985,14 @@
       </c>
       <c r="C8" s="44">
         <f t="shared" ca="1" si="0"/>
-        <v>530</v>
+        <v>994</v>
       </c>
       <c r="F8" s="45" t="s">
         <v>47</v>
       </c>
       <c r="G8" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F8, $C$2:$C$9)</f>
-        <v>1607</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -6293,14 +7004,14 @@
       </c>
       <c r="C9" s="42">
         <f t="shared" ca="1" si="0"/>
-        <v>902</v>
+        <v>761</v>
       </c>
       <c r="F9" s="34" t="s">
         <v>50</v>
       </c>
       <c r="G9" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F9)</f>
-        <v>902</v>
+        <v>960</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -6309,7 +7020,7 @@
       </c>
       <c r="G10" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F8, $B$2:$B$9, F10)</f>
-        <v>705</v>
+        <v>822</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -6318,7 +7029,7 @@
       </c>
       <c r="G11" s="46">
         <f ca="1">SUMIF($A$2:$A$9, F11, $C$2:$C$9)</f>
-        <v>1432</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -6327,7 +7038,7 @@
       </c>
       <c r="G12" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F12)</f>
-        <v>530</v>
+        <v>994</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -6336,7 +7047,7 @@
       </c>
       <c r="G13" s="34">
         <f ca="1">SUMIFS($C$2:$C$9, $A$2:$A$9, F11, $B$2:$B$9, F13)</f>
-        <v>902</v>
+        <v>761</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -6345,7 +7056,7 @@
       </c>
       <c r="G14" s="43">
         <f ca="1">SUM(G2,G5,G8,G11)</f>
-        <v>5669</v>
+        <v>6526</v>
       </c>
     </row>
   </sheetData>
@@ -6530,10 +7241,10 @@
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C12" s="80" t="s">
+      <c r="C12" s="82" t="s">
         <v>74</v>
       </c>
-      <c r="D12" s="80"/>
+      <c r="D12" s="82"/>
       <c r="E12" s="66">
         <f>SUM(JLoka_Investors[INVESTMENT AMOUNT (USD)])</f>
         <v>180500</v>
@@ -6572,12 +7283,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B2" s="81" t="s">
+      <c r="B2" s="83" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
       <c r="F2" s="67"/>
     </row>
     <row r="3" spans="2:6" s="67" customFormat="1" x14ac:dyDescent="0.25">
@@ -6600,15 +7311,15 @@
       </c>
       <c r="C4" s="3">
         <f ca="1">RAND()</f>
-        <v>0.1970140427985092</v>
+        <v>0.16531561844993903</v>
       </c>
       <c r="D4" s="3">
         <f t="shared" ref="D4:E4" ca="1" si="0">RAND()</f>
-        <v>0.61752950258084438</v>
+        <v>0.95530460667608263</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.59433522503123093</v>
+        <v>9.1390388979077919E-3</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -6617,15 +7328,15 @@
       </c>
       <c r="C5" s="3">
         <f t="shared" ref="C5:E14" ca="1" si="1">RAND()</f>
-        <v>0.6633830799647159</v>
+        <v>0.18240848603514137</v>
       </c>
       <c r="D5" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.52714726800078981</v>
+        <v>7.4365587247146259E-2</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.69668174009225037</v>
+        <v>0.44820563268627189</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
@@ -6634,15 +7345,15 @@
       </c>
       <c r="C6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.17562438708328187</v>
+        <v>0.56155399528444627</v>
       </c>
       <c r="D6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.9163764591219179</v>
+        <v>0.68186447037085673</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.98052310491075534</v>
+        <v>0.22676712201392224</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
@@ -6651,15 +7362,15 @@
       </c>
       <c r="C7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.97179011742401034</v>
+        <v>0.52126929017846724</v>
       </c>
       <c r="D7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.86700995900552902</v>
+        <v>0.60875095923928202</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.53703235256206727</v>
+        <v>0.84204372880442302</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
@@ -6668,15 +7379,15 @@
       </c>
       <c r="C8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.84749572115146177</v>
+        <v>0.97925953918999264</v>
       </c>
       <c r="D8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.14018279942935719</v>
+        <v>0.88291092579954622</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.16890054256540799</v>
+        <v>0.45790128096059224</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
@@ -6685,15 +7396,15 @@
       </c>
       <c r="C9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.93566798383572247</v>
+        <v>0.10034826295175892</v>
       </c>
       <c r="D9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.92855436625288845</v>
+        <v>0.58665416372055923</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.1460052583933078</v>
+        <v>0.36038891406072593</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
@@ -6702,15 +7413,15 @@
       </c>
       <c r="C10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.1433999468745274</v>
+        <v>0.9503281952830277</v>
       </c>
       <c r="D10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.63410830731845791</v>
+        <v>0.33359262369764586</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.6021723468059248</v>
+        <v>0.75719536474901727</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
@@ -6719,15 +7430,15 @@
       </c>
       <c r="C11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.21221459352036331</v>
+        <v>0.87703057541907758</v>
       </c>
       <c r="D11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.30477536836824548</v>
+        <v>0.80630794943668815</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>5.9313688358269889E-2</v>
+        <v>0.15921596559988871</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
@@ -6736,15 +7447,15 @@
       </c>
       <c r="C12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>4.7972957196397492E-2</v>
+        <v>0.80006013547308241</v>
       </c>
       <c r="D12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.63336008174203462</v>
+        <v>0.52751584656207184</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.19399467707450213</v>
+        <v>0.92639734750661817</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
@@ -6753,15 +7464,15 @@
       </c>
       <c r="C13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.72753524488705212</v>
+        <v>0.28464794699125118</v>
       </c>
       <c r="D13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.44769928553516947</v>
+        <v>0.39156857781522625</v>
       </c>
       <c r="E13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.22340416548027076</v>
+        <v>0.52483943302404878</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
@@ -6770,15 +7481,15 @@
       </c>
       <c r="C14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.89667820846322988</v>
+        <v>0.29989699726608532</v>
       </c>
       <c r="D14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.3584885461089784</v>
+        <v>0.19502874159617778</v>
       </c>
       <c r="E14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>6.1928356350029135E-2</v>
+        <v>0.57672047294585982</v>
       </c>
     </row>
   </sheetData>

</xml_diff>